<commit_message>
Add collapsed core, stream uplink headroom and 1G router fallback
- A single main-room switch with free ports for every closet link is also
  the core, so small designs need no separate core switch; the diagram
  shows the main room in the core position with the links it terminates
- Replace the 10G minimum uplink with a stream-basis headroom margin
  (Stream_Uplink_Headroom_Pct, 50%); Min_Uplink_Gbps back to 1, so audio
  on stream bandwidth uses 1G switches and 1G uplinks
- Router falls back to a free 1G copper port, then a 1G SFP module
  (AGM731F, to be confirmed on the PR460X), with an alert in Checks
- Count the router port in the switch gauge; straight labelled router
  line for a standalone switch
- Add validation scenarios V26-V30 and regenerate the reports
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1171,7 +1171,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:C22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C22"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Area"/>
@@ -1222,7 +1222,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCompat" displayName="tblCompat" ref="A4:G171" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCompat" displayName="tblCompat" ref="A4:G172" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:G171"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Scope_Type"/>
@@ -1308,7 +1308,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Key"/>
@@ -2693,7 +2693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="28" min="1" max="1"/>
@@ -2902,78 +2902,95 @@
       </c>
       <c r="B15" s="43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" s="43" t="inlineStr">
         <is>
-          <t>Slowest uplink speed to the core. 10 keeps headroom even when only audio or control devices are in a room; 1 allows 1G uplinks</t>
+          <t>Slowest uplink speed to the core. 1 allows 1G uplinks when the bandwidth fits (for example audio on stream bandwidth); raise to 10 to force 10G uplinks everywhere</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
         <is>
-          <t>Uplink_LAG_Sizes</t>
+          <t>Stream_Uplink_Headroom_Pct</t>
         </is>
       </c>
       <c r="B16" s="43" t="inlineStr">
         <is>
-          <t>1,2,4,8</t>
-        </is>
-      </c>
-      <c r="C16" s="51" t="inlineStr">
-        <is>
-          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Stream bandwidth basis only: uplinks must carry the stream total plus this margin, because stream rates are typical, not peak. Line-rate needs no margin</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
         <is>
-          <t>In_Rack_Max_m</t>
+          <t>Uplink_LAG_Sizes</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C17" s="43" t="inlineStr">
-        <is>
-          <t>MDF links at or below this use DAC/AOC</t>
+          <t>1,2,4,8</t>
+        </is>
+      </c>
+      <c r="C17" s="51" t="inlineStr">
+        <is>
+          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
         <is>
-          <t>Copper_10G_Max_m</t>
+          <t>In_Rack_Max_m</t>
         </is>
       </c>
       <c r="B18" s="43" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C18" s="43" t="inlineStr">
         <is>
-          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+          <t>MDF links at or below this use DAC/AOC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
         <is>
+          <t>Copper_10G_Max_m</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
           <t>Endpoint_Speeds_Gbps</t>
         </is>
       </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="B20" s="43" t="inlineStr">
         <is>
           <t>1,2.5,5,10,25,50,100</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C20" s="43" t="inlineStr">
         <is>
           <t>Speeds offered in the endpoint library</t>
         </is>
@@ -6344,7 +6361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -6686,6 +6703,23 @@
       <c r="C22" s="51" t="inlineStr">
         <is>
           <t>AXM761 (10G SR) assumed on both ends. Confirm the validated optic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
+          <t>PR460X</t>
+        </is>
+      </c>
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t>1G SFP (AGM731F) in the PR460X SFP+ port is not confirmed in the datasheet.</t>
+        </is>
+      </c>
+      <c r="C23" s="51" t="inlineStr">
+        <is>
+          <t>Allowed as a last-resort 1G router link with a warning. Confirm with PLM.</t>
         </is>
       </c>
     </row>
@@ -29723,7 +29757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G171"/>
+  <dimension ref="A1:G172"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="28" min="1" max="1"/>
@@ -35348,6 +35382,39 @@
       <c r="G171" s="43" t="inlineStr">
         <is>
           <t>DAC and AOC cables are not compatible with the PR460X SFP+ port</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B172" s="43" t="inlineStr">
+        <is>
+          <t>PR460X</t>
+        </is>
+      </c>
+      <c r="C172" s="43" t="inlineStr">
+        <is>
+          <t>SFP+ (10G LAN)</t>
+        </is>
+      </c>
+      <c r="D172" s="43" t="inlineStr">
+        <is>
+          <t>AGM731F</t>
+        </is>
+      </c>
+      <c r="E172" s="43" t="inlineStr">
+        <is>
+          <t>Optional optic (1G, to confirm)</t>
+        </is>
+      </c>
+      <c r="F172" s="43" t="n"/>
+      <c r="G172" s="43" t="inlineStr">
+        <is>
+          <t>Used only when no 10G port is free: 1G SX module on both ends. Confirm the PR460X SFP+ port accepts 1G modules</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace OnCall with Sprint, Overdrive and Fastlane support contracts
- Catalog: Support_Tiers and Included_Support per product, SKU pattern
  {tier}-{Product_ID}-{months} (SPR / DRV / FLS) from the Support 2.0
  update; OnCall PMB03 rows marked legacy; open questions in Data_Gaps
- Support contract option lists only tiers offered for the products in the
  design, 1/3/5 years; SKUs for switches, access points and the router
- Sprint up to the included 3 years adds no SKU for managed switches;
  tiers a product does not offer give a warning instead of a SKU
- Older projects with OnCall years open as Overdrive for the same term
- Add validation scenarios V33 and V34
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1058,9 +1058,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CM38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CO38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:CM38"/>
-  <tableColumns count="91">
+  <tableColumns count="93">
     <tableColumn id="1" name="Product_ID"/>
     <tableColumn id="2" name="Model_Name"/>
     <tableColumn id="3" name="Family"/>
@@ -1152,12 +1152,14 @@
     <tableColumn id="89" name="Source_Datasheet"/>
     <tableColumn id="90" name="Last_Verified"/>
     <tableColumn id="91" name="Data_Notes"/>
+    <tableColumn id="92" name="Support_Tiers"/>
+    <tableColumn id="93" name="Included_Support"/>
   </tableColumns>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F116" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F113"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Sheet"/>
@@ -1171,7 +1173,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C22"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Area"/>
@@ -2808,12 +2810,12 @@
       </c>
       <c r="B9" s="43" t="inlineStr">
         <is>
-          <t>PMB03{years}{cat}-10000S</t>
+          <t>{tier}-{pid}-{months}</t>
         </is>
       </c>
       <c r="C9" s="51" t="inlineStr">
         <is>
-          <t>{years}=1/3/5, {cat}=digit from Support_Category</t>
+          <t>tier = SPR (Sprint), DRV (Overdrive), FLS (Fastlane); pid = Product_ID; months = 12/36/60. Source: Confluence SSO "Support 2.0 Update" (Apr 2026)</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="28" min="1" max="1"/>
@@ -6338,6 +6340,54 @@
       <c r="F114" s="51" t="inlineStr">
         <is>
           <t>Blank = any switch. 'PTP-BC' = needs PTP boundary clock (room switch and core). 'AVB' = needs AVB; M4250 gets one uplink per core (no LAG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="43" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B115" s="51" t="inlineStr">
+        <is>
+          <t>Support_Tiers</t>
+        </is>
+      </c>
+      <c r="C115" s="43" t="n"/>
+      <c r="D115" s="43" t="n"/>
+      <c r="E115" s="43" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="F115" s="51" t="inlineStr">
+        <is>
+          <t>Support tiers that can be bought: Sprint, Overdrive, Fastlane. The tool offers only these per product</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="43" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B116" s="51" t="inlineStr">
+        <is>
+          <t>Included_Support</t>
+        </is>
+      </c>
+      <c r="C116" s="43" t="n"/>
+      <c r="D116" s="43" t="n"/>
+      <c r="E116" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F116" s="51" t="inlineStr">
+        <is>
+          <t>Support included with the product, e.g. 'Sprint 3 yr' for managed switches (no SKU needed)</t>
         </is>
       </c>
     </row>
@@ -6361,7 +6411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -6720,6 +6770,40 @@
       <c r="C23" s="51" t="inlineStr">
         <is>
           <t>Allowed as a last-resort 1G router link with a warning. Confirm with PLM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>Sprint / Overdrive / Fastlane SKUs ({tier}-{Product_ID}-{12/36/60}) follow the pattern in Confluence SSO "Support 2.0 Update" (Apr 2026); per-model SKUs are not listed in the datasheets.</t>
+        </is>
+      </c>
+      <c r="C24" s="51" t="inlineStr">
+        <is>
+          <t>Confirm the SKU exists for each model before quoting. Fastlane confirmed on reseller listings for M4350; to confirm for M4250.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="43" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>Fastlane for M4500, WBE718/758 and PR460X is not listed in their datasheets.</t>
+        </is>
+      </c>
+      <c r="C25" s="51" t="inlineStr">
+        <is>
+          <t>Support_Tiers set to Sprint, Overdrive for these. Add Fastlane when confirmed.</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CM38"/>
+  <dimension ref="A1:CO38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -7204,6 +7288,8 @@
     <col width="28" customWidth="1" style="28" min="89" max="89"/>
     <col width="11" customWidth="1" style="28" min="90" max="90"/>
     <col width="40" customWidth="1" style="28" min="91" max="91"/>
+    <col width="26" customWidth="1" style="29" min="92" max="92"/>
+    <col width="26" customWidth="1" style="29" min="93" max="93"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -7825,6 +7911,16 @@
           <t>Data_Notes</t>
         </is>
       </c>
+      <c r="CN4" s="42" t="inlineStr">
+        <is>
+          <t>Support_Tiers</t>
+        </is>
+      </c>
+      <c r="CO4" s="42" t="inlineStr">
+        <is>
+          <t>Included_Support</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" s="29">
       <c r="A5" s="43" t="inlineStr">
@@ -8125,6 +8221,16 @@
           <t>Throughput 14.88 Mpps (perf table) vs 14.80 Mpps (spec table) - verify</t>
         </is>
       </c>
+      <c r="CN5" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO5" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="46.25" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -8421,6 +8527,16 @@
         </is>
       </c>
       <c r="CM6" s="43" t="n"/>
+      <c r="CN6" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO6" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="46.25" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -8719,6 +8835,16 @@
         </is>
       </c>
       <c r="CM7" s="43" t="n"/>
+      <c r="CN7" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO7" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="46.25" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -9017,6 +9143,16 @@
         </is>
       </c>
       <c r="CM8" s="43" t="n"/>
+      <c r="CN8" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO8" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="46.25" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -9315,6 +9451,16 @@
         </is>
       </c>
       <c r="CM9" s="43" t="n"/>
+      <c r="CN9" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO9" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="46.25" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -9613,6 +9759,16 @@
         </is>
       </c>
       <c r="CM10" s="43" t="n"/>
+      <c r="CN10" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO10" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="46.25" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -9915,6 +10071,16 @@
           <t>PoE budget 720W with 1 PSU powered, 1,440W with 2. Full-PoE power: 889W (1 PSU) / 1,734W (2 PSU)</t>
         </is>
       </c>
+      <c r="CN11" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO11" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="46.25" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -10213,6 +10379,16 @@
         </is>
       </c>
       <c r="CM12" s="43" t="n"/>
+      <c r="CN12" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO12" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="46.25" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -10511,6 +10687,16 @@
         </is>
       </c>
       <c r="CM13" s="43" t="n"/>
+      <c r="CN13" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO13" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="46.25" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -10809,6 +10995,16 @@
         </is>
       </c>
       <c r="CM14" s="43" t="n"/>
+      <c r="CN14" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO14" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="46.25" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -11111,6 +11307,16 @@
           <t>PoE budget 720W (1 PSU) / 1,650W (2 PSU) / 2,880W (3 PSU). Full-PoE power: 912 / 1,998 / 3,523W</t>
         </is>
       </c>
+      <c r="CN15" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO15" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="46.25" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -11400,6 +11606,16 @@
         </is>
       </c>
       <c r="CM16" s="43" t="n"/>
+      <c r="CN16" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO16" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="46.25" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -11699,6 +11915,16 @@
           <t>Weight: 1.74 kg on product page vs 2.80 kg in spec table - verify</t>
         </is>
       </c>
+      <c r="CN17" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO17" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="46.25" customHeight="1" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -11999,6 +12225,16 @@
         </is>
       </c>
       <c r="CM18" s="43" t="n"/>
+      <c r="CN18" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO18" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="46.25" customHeight="1" s="29">
       <c r="A19" s="43" t="inlineStr">
@@ -12299,6 +12535,16 @@
         </is>
       </c>
       <c r="CM19" s="43" t="n"/>
+      <c r="CN19" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO19" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46.25" customHeight="1" s="29">
       <c r="A20" s="43" t="inlineStr">
@@ -12607,6 +12853,16 @@
           <t>Ships with 1x APS254W. Redundant budget 119W (1+1) or 322W (2+1). Optional PST4310 half-width PSU tray.</t>
         </is>
       </c>
+      <c r="CN20" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO20" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="46.25" customHeight="1" s="29">
       <c r="A21" s="43" t="inlineStr">
@@ -12911,6 +13167,16 @@
         </is>
       </c>
       <c r="CM21" s="43" t="n"/>
+      <c r="CN21" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO21" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="46.25" customHeight="1" s="29">
       <c r="A22" s="43" t="inlineStr">
@@ -13219,6 +13485,16 @@
           <t>Max 3,314W PoE needs 2x APS2000W on 220VAC</t>
         </is>
       </c>
+      <c r="CN22" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO22" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="46.25" customHeight="1" s="29">
       <c r="A23" s="43" t="inlineStr">
@@ -13516,6 +13792,16 @@
           <t>Modular slot = RPS only (no PoE)</t>
         </is>
       </c>
+      <c r="CN23" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO23" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="46.25" customHeight="1" s="29">
       <c r="A24" s="43" t="inlineStr">
@@ -13809,6 +14095,16 @@
         </is>
       </c>
       <c r="CM24" s="43" t="n"/>
+      <c r="CN24" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO24" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="46.25" customHeight="1" s="29">
       <c r="A25" s="43" t="inlineStr">
@@ -14102,6 +14398,16 @@
         </is>
       </c>
       <c r="CM25" s="43" t="n"/>
+      <c r="CN25" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO25" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="46.25" customHeight="1" s="29">
       <c r="A26" s="43" t="inlineStr">
@@ -14406,6 +14712,16 @@
         </is>
       </c>
       <c r="CM26" s="43" t="n"/>
+      <c r="CN26" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO26" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="46.25" customHeight="1" s="29">
       <c r="A27" s="43" t="inlineStr">
@@ -14703,6 +15019,16 @@
           <t>Modular slot = RPS only (no PoE)</t>
         </is>
       </c>
+      <c r="CN27" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO27" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="46.25" customHeight="1" s="29">
       <c r="A28" s="43" t="inlineStr">
@@ -15007,6 +15333,16 @@
         </is>
       </c>
       <c r="CM28" s="43" t="n"/>
+      <c r="CN28" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO28" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="46.25" customHeight="1" s="29">
       <c r="A29" s="43" t="inlineStr">
@@ -15311,6 +15647,16 @@
         </is>
       </c>
       <c r="CM29" s="43" t="n"/>
+      <c r="CN29" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO29" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="46.25" customHeight="1" s="29">
       <c r="A30" s="43" t="inlineStr">
@@ -15608,6 +15954,16 @@
           <t>Modular slot = RPS only (no PoE)</t>
         </is>
       </c>
+      <c r="CN30" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO30" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="46.25" customHeight="1" s="29">
       <c r="A31" s="43" t="inlineStr">
@@ -15905,6 +16261,16 @@
           <t>Modular slot = RPS only (no PoE)</t>
         </is>
       </c>
+      <c r="CN31" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO31" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="29">
       <c r="A32" s="43" t="inlineStr">
@@ -16209,6 +16575,16 @@
         </is>
       </c>
       <c r="CM32" s="43" t="n"/>
+      <c r="CN32" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO32" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="29">
       <c r="A33" s="43" t="inlineStr">
@@ -16506,6 +16882,16 @@
           <t>Modular slot = RPS only (no PoE)</t>
         </is>
       </c>
+      <c r="CN33" s="43" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO33" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="57.45" customHeight="1" s="29">
       <c r="A34" s="43" t="inlineStr">
@@ -16774,6 +17160,12 @@
           <t>Concurrent connections: 60,000 (spec table) vs 250,000 (features table) - verify. Optional Exium security license (SEC-PR460X-xx), Insight path only.</t>
         </is>
       </c>
+      <c r="CN34" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive</t>
+        </is>
+      </c>
+      <c r="CO34" s="51" t="n"/>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="29">
       <c r="A35" s="43" t="inlineStr">
@@ -17028,6 +17420,12 @@
           <t>Weight shown as 0.69 kg (2.09 lb) - lb value inconsistent, verify. Engage support per PR460X datasheet ('select APs') - confirm model list.</t>
         </is>
       </c>
+      <c r="CN35" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive</t>
+        </is>
+      </c>
+      <c r="CO35" s="51" t="n"/>
     </row>
     <row r="36" ht="46.25" customHeight="1" s="29">
       <c r="A36" s="43" t="inlineStr">
@@ -17282,6 +17680,12 @@
           <t>Datasheet intro says 7.8 Gbps, spec table 18.4 Gbps - verify. 2.4GHz listed as 802.11b/g/n/ax (no be).</t>
         </is>
       </c>
+      <c r="CN36" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive</t>
+        </is>
+      </c>
+      <c r="CO36" s="51" t="n"/>
     </row>
     <row r="37" ht="46.25" customHeight="1" s="29">
       <c r="A37" s="43" t="inlineStr">
@@ -17577,6 +17981,16 @@
           <t>Spine for M4500-48XF8C leaf switches (datasheet: 320 x 320 at 10G). Acoustic value is the 25C figure, not a quiet mode. Datasheet lists no AVB or PTP boundary clock.</t>
         </is>
       </c>
+      <c r="CN37" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive</t>
+        </is>
+      </c>
+      <c r="CO37" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="46.25" customHeight="1" s="29">
       <c r="A38" s="43" t="inlineStr">
@@ -17872,11 +18286,21 @@
           <t>Leaf (10G/25G access) or core for many 10G/25G links. Acoustic value is the 25C figure. Datasheet lists no AVB or PTP boundary clock.</t>
         </is>
       </c>
+      <c r="CN38" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive</t>
+        </is>
+      </c>
+      <c r="CO38" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:CM2"/>
-    <mergeCell ref="A1:CM1"/>
+    <mergeCell ref="A1:CO1"/>
+    <mergeCell ref="A2:CO2"/>
   </mergeCells>
   <dataValidations count="8">
     <dataValidation sqref="E5:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
@@ -25570,7 +25994,11 @@
           <t>M4250 datasheet DS-M4250-9Nov23 (fw 13.0.4)</t>
         </is>
       </c>
-      <c r="Q50" s="43" t="n"/>
+      <c r="Q50" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="23.85" customHeight="1" s="29">
       <c r="A51" s="43" t="inlineStr">
@@ -25611,7 +26039,11 @@
           <t>M4250 datasheet DS-M4250-9Nov23 (fw 13.0.4)</t>
         </is>
       </c>
-      <c r="Q51" s="43" t="n"/>
+      <c r="Q51" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="23.85" customHeight="1" s="29">
       <c r="A52" s="43" t="inlineStr">
@@ -25652,7 +26084,11 @@
           <t>M4250 datasheet DS-M4250-9Nov23 (fw 13.0.4)</t>
         </is>
       </c>
-      <c r="Q52" s="43" t="n"/>
+      <c r="Q52" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="29">
       <c r="A53" s="43" t="inlineStr">
@@ -25693,7 +26129,11 @@
           <t>M4250 + M4350 datasheets</t>
         </is>
       </c>
-      <c r="Q53" s="43" t="n"/>
+      <c r="Q53" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="29">
       <c r="A54" s="43" t="inlineStr">
@@ -25734,7 +26174,11 @@
           <t>M4250 + M4350 datasheets</t>
         </is>
       </c>
-      <c r="Q54" s="43" t="n"/>
+      <c r="Q54" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="29">
       <c r="A55" s="43" t="inlineStr">
@@ -25775,7 +26219,11 @@
           <t>M4250 + M4350 datasheets</t>
         </is>
       </c>
-      <c r="Q55" s="43" t="n"/>
+      <c r="Q55" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="46.25" customHeight="1" s="29">
       <c r="A56" s="43" t="inlineStr">
@@ -25816,7 +26264,11 @@
           <t>M4350 datasheet DS-M4350-30May25 (fw 14.0) [file: M3450_Datasheet_30May25.pdf]</t>
         </is>
       </c>
-      <c r="Q56" s="43" t="n"/>
+      <c r="Q56" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="46.25" customHeight="1" s="29">
       <c r="A57" s="43" t="inlineStr">
@@ -25857,7 +26309,11 @@
           <t>M4350 datasheet DS-M4350-30May25 (fw 14.0) [file: M3450_Datasheet_30May25.pdf]</t>
         </is>
       </c>
-      <c r="Q57" s="43" t="n"/>
+      <c r="Q57" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="46.25" customHeight="1" s="29">
       <c r="A58" s="43" t="inlineStr">
@@ -25898,7 +26354,11 @@
           <t>M4350 datasheet DS-M4350-30May25 (fw 14.0) [file: M3450_Datasheet_30May25.pdf]</t>
         </is>
       </c>
-      <c r="Q58" s="43" t="n"/>
+      <c r="Q58" s="43" t="inlineStr">
+        <is>
+          <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="29">
       <c r="A59" s="43" t="inlineStr">

</xml_diff>

<commit_message>
Add M4350-16C and M4350-16M4V, Neutrik rooms and ST 2110-30 audio
- Catalog from DS-M4350-03Jul26: M4350-16C (16 x 100G, boundary clock)
  and M4350-16M4V (Neutrik etherCON, 1+1 internal PSUs) with SKUs, PSU
  rows, APM414V/C/SD/LD interface cards and design rules
- New Neutrik_etherCON_Ports column; rooms get a Connectors setting, and
  Neutrik switches are only used in Neutrik rooms (never as a core)
- New ST 2110-30 / AES67 audio device type (PTP boundary clock)
- Data_Gaps: datasheet lists Sprint/Overdrive SKUs only; cards beyond
  APM414V not chosen by the tool yet
- Add validation scenarios V35-V37 and regenerate the reports
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1058,9 +1058,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CO38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CP40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:CM38"/>
-  <tableColumns count="93">
+  <tableColumns count="94">
     <tableColumn id="1" name="Product_ID"/>
     <tableColumn id="2" name="Model_Name"/>
     <tableColumn id="3" name="Family"/>
@@ -1154,12 +1154,13 @@
     <tableColumn id="91" name="Data_Notes"/>
     <tableColumn id="92" name="Support_Tiers"/>
     <tableColumn id="93" name="Included_Support"/>
+    <tableColumn id="94" name="Neutrik_etherCON_Ports"/>
   </tableColumns>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F116" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F113"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Sheet"/>
@@ -1173,7 +1174,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="tblGaps" displayName="tblGaps" ref="A4:F27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C22"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Area"/>
@@ -1184,7 +1185,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblSKUs" displayName="tblSKUs" ref="A4:G149" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblSKUs" displayName="tblSKUs" ref="A4:G157" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:G149"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Product_ID"/>
@@ -1199,7 +1200,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:Q127" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:Q131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:Q127"/>
   <tableColumns count="17">
     <tableColumn id="1" name="Orderable_SKU"/>
@@ -1224,7 +1225,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCompat" displayName="tblCompat" ref="A4:G172" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCompat" displayName="tblCompat" ref="A4:G176" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:G171"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Scope_Type"/>
@@ -1239,7 +1240,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblPSUMatrix" displayName="tblPSUMatrix" ref="A4:L107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblPSUMatrix" displayName="tblPSUMatrix" ref="A4:L115" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:L107"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Product_ID"/>
@@ -1259,7 +1260,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblRules" displayName="tblRules" ref="A4:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblRules" displayName="tblRules" ref="A4:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F23"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Rule_ID"/>
@@ -1273,7 +1274,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblEndpoints" displayName="tblEndpoints" ref="A4:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblEndpoints" displayName="tblEndpoints" ref="A4:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:J18"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Endpoint_ID"/>
@@ -1838,7 +1839,7 @@
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>M4250: DS-M4250-9Nov23 · M4350: DS-M4350-30May25 (uploaded as 'M3450_Datasheet_30May25.pdf') · PR460X: NG_DS_AV_PR460X-042926 · WBE718: DS-WBE718_02Apr26 · WBE758: D-WBE758_29Jan24 · 25G/100G optics &amp; DACs: optic.ca, NETGEAR KB 000066694 (updated 2025-09-23) · M4500: DS-M4500-3Apr26</t>
+          <t>M4250: DS-M4250-9Nov23 · M4350: DS-M4350-30May25 (uploaded as 'M3450_Datasheet_30May25.pdf') · PR460X: NG_DS_AV_PR460X-042926 · WBE718: DS-WBE718_02Apr26 · WBE758: D-WBE758_29Jan24 · 25G/100G optics &amp; DACs: optic.ca, NETGEAR KB 000066694 (updated 2025-09-23) · M4500: DS-M4500-3Apr26 · M4350-16C/16M4V: DS-M4350-03Jul26</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2743,7 @@
       </c>
       <c r="B5" s="43" t="inlineStr">
         <is>
-          <t>2026.10.01b</t>
+          <t>2026.10.01c</t>
         </is>
       </c>
       <c r="C5" s="43" t="inlineStr">
@@ -3018,7 +3019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="28" min="1" max="1"/>
@@ -6367,7 +6368,7 @@
         </is>
       </c>
     </row>
-    <row r="116">
+    <row r="116" s="29">
       <c r="A116" s="43" t="inlineStr">
         <is>
           <t>Products</t>
@@ -6388,6 +6389,34 @@
       <c r="F116" s="51" t="inlineStr">
         <is>
           <t>Support included with the product, e.g. 'Sprint 3 yr' for managed switches (no SKU needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="43" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B117" s="51" t="inlineStr">
+        <is>
+          <t>Neutrik_etherCON_Ports</t>
+        </is>
+      </c>
+      <c r="C117" s="43" t="n"/>
+      <c r="D117" s="43" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E117" s="43" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="F117" s="51" t="inlineStr">
+        <is>
+          <t>Locking Neutrik etherCON RJ45 ports (front). 0 = standard RJ45 only</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -6790,7 +6819,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" s="29">
       <c r="A25" s="43" t="inlineStr">
         <is>
           <t>Support</t>
@@ -6804,6 +6833,40 @@
       <c r="C25" s="51" t="inlineStr">
         <is>
           <t>Support_Tiers set to Sprint, Overdrive for these. Add Fastlane when confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>M4350</t>
+        </is>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>Datasheet DS-M4350-03Jul26 lists Sprint and Overdrive SKUs per model; Fastlane is not listed.</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="inlineStr">
+        <is>
+          <t>Fastlane kept as an option per the Support 2.0 update (bought through resellers). Confirm per model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>Interface card options (APM414C/SD/LD) are in the catalog but the tool always assumes the shipping APM414V card.</t>
+        </is>
+      </c>
+      <c r="C27" s="51" t="inlineStr">
+        <is>
+          <t>Card choice to be added to the tool.</t>
         </is>
       </c>
     </row>
@@ -6827,7 +6890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="28" min="1" max="11"/>
@@ -7199,6 +7262,13 @@
       <c r="H17" s="39" t="inlineStr">
         <is>
           <t>Fan Tray</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="H18" s="39" t="inlineStr">
+        <is>
+          <t>Interface Card</t>
         </is>
       </c>
     </row>
@@ -7219,7 +7289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CO38"/>
+  <dimension ref="A1:CP40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -7290,6 +7360,7 @@
     <col width="40" customWidth="1" style="28" min="91" max="91"/>
     <col width="26" customWidth="1" style="29" min="92" max="92"/>
     <col width="26" customWidth="1" style="29" min="93" max="93"/>
+    <col width="14" customWidth="1" style="29" min="94" max="94"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -7921,6 +7992,11 @@
           <t>Included_Support</t>
         </is>
       </c>
+      <c r="CP4" s="42" t="inlineStr">
+        <is>
+          <t>Neutrik_etherCON_Ports</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="46.25" customHeight="1" s="29">
       <c r="A5" s="43" t="inlineStr">
@@ -8231,6 +8307,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP5" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="46.25" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -8537,6 +8616,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP6" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="46.25" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -8845,6 +8927,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP7" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="46.25" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -9153,6 +9238,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP8" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="46.25" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -9461,6 +9549,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP9" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="46.25" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -9769,6 +9860,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP10" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="46.25" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -10081,6 +10175,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP11" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="46.25" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -10389,6 +10486,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP12" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="46.25" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -10697,6 +10797,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP13" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="46.25" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -11005,6 +11108,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP14" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="46.25" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -11317,6 +11423,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP15" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" ht="46.25" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -11616,6 +11725,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP16" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="46.25" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -11925,6 +12037,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP17" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="46.25" customHeight="1" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -12235,6 +12350,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP18" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="46.25" customHeight="1" s="29">
       <c r="A19" s="43" t="inlineStr">
@@ -12545,6 +12663,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP19" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="46.25" customHeight="1" s="29">
       <c r="A20" s="43" t="inlineStr">
@@ -12863,6 +12984,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP20" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="46.25" customHeight="1" s="29">
       <c r="A21" s="43" t="inlineStr">
@@ -13177,6 +13301,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP21" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" ht="46.25" customHeight="1" s="29">
       <c r="A22" s="43" t="inlineStr">
@@ -13495,6 +13622,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP22" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" ht="46.25" customHeight="1" s="29">
       <c r="A23" s="43" t="inlineStr">
@@ -13802,6 +13932,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP23" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="46.25" customHeight="1" s="29">
       <c r="A24" s="43" t="inlineStr">
@@ -14105,6 +14238,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP24" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="46.25" customHeight="1" s="29">
       <c r="A25" s="43" t="inlineStr">
@@ -14408,6 +14544,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP25" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" ht="46.25" customHeight="1" s="29">
       <c r="A26" s="43" t="inlineStr">
@@ -14722,6 +14861,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP26" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="46.25" customHeight="1" s="29">
       <c r="A27" s="43" t="inlineStr">
@@ -15029,6 +15171,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP27" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" ht="46.25" customHeight="1" s="29">
       <c r="A28" s="43" t="inlineStr">
@@ -15343,6 +15488,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP28" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" ht="46.25" customHeight="1" s="29">
       <c r="A29" s="43" t="inlineStr">
@@ -15657,6 +15805,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP29" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" ht="46.25" customHeight="1" s="29">
       <c r="A30" s="43" t="inlineStr">
@@ -15964,6 +16115,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP30" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" ht="46.25" customHeight="1" s="29">
       <c r="A31" s="43" t="inlineStr">
@@ -16271,6 +16425,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP31" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="29">
       <c r="A32" s="43" t="inlineStr">
@@ -16585,6 +16742,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP32" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="29">
       <c r="A33" s="43" t="inlineStr">
@@ -16892,6 +17052,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP33" s="43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" ht="57.45" customHeight="1" s="29">
       <c r="A34" s="43" t="inlineStr">
@@ -17166,6 +17329,9 @@
         </is>
       </c>
       <c r="CO34" s="51" t="n"/>
+      <c r="CP34" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="29">
       <c r="A35" s="43" t="inlineStr">
@@ -17426,6 +17592,9 @@
         </is>
       </c>
       <c r="CO35" s="51" t="n"/>
+      <c r="CP35" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" ht="46.25" customHeight="1" s="29">
       <c r="A36" s="43" t="inlineStr">
@@ -17686,6 +17855,9 @@
         </is>
       </c>
       <c r="CO36" s="51" t="n"/>
+      <c r="CP36" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="46.25" customHeight="1" s="29">
       <c r="A37" s="43" t="inlineStr">
@@ -17991,6 +18163,9 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP37" s="51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" ht="46.25" customHeight="1" s="29">
       <c r="A38" s="43" t="inlineStr">
@@ -18296,11 +18471,645 @@
           <t>Sprint 3 yr</t>
         </is>
       </c>
+      <c r="CP38" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" ht="46.25" customHeight="1" s="29">
+      <c r="A39" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B39" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C39" s="43" t="inlineStr">
+        <is>
+          <t>M4350</t>
+        </is>
+      </c>
+      <c r="D39" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR AV and IT</t>
+        </is>
+      </c>
+      <c r="E39" s="43" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F39" s="43" t="inlineStr">
+        <is>
+          <t>Aggregation / Core</t>
+        </is>
+      </c>
+      <c r="G39" s="43" t="inlineStr">
+        <is>
+          <t>AV UI; Engage; IT Web GUI; CLI; SNMP</t>
+        </is>
+      </c>
+      <c r="H39" s="43" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I39" s="44" t="n"/>
+      <c r="J39" s="45" t="n"/>
+      <c r="K39" s="45" t="n"/>
+      <c r="L39" s="43" t="inlineStr">
+        <is>
+          <t>1U rack</t>
+        </is>
+      </c>
+      <c r="M39" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" s="43" t="inlineStr">
+        <is>
+          <t>Full width</t>
+        </is>
+      </c>
+      <c r="O39" s="43" t="n">
+        <v>440</v>
+      </c>
+      <c r="P39" s="43" t="n">
+        <v>400</v>
+      </c>
+      <c r="Q39" s="43" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="R39" s="46" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="S39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="43" t="n">
+        <v>16</v>
+      </c>
+      <c r="AA39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF39" s="47">
+        <f>SUM(S39:AE39)</f>
+        <v>16</v>
+      </c>
+      <c r="AG39" s="43" t="n"/>
+      <c r="AH39" s="43" t="inlineStr">
+        <is>
+          <t>QSFP28: 40G or 100G (stacking 100G only). No 10G/25G without breakout</t>
+        </is>
+      </c>
+      <c r="AI39" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AK39" s="43" t="n"/>
+      <c r="AL39" s="48" t="n"/>
+      <c r="AM39" s="48" t="n"/>
+      <c r="AN39" s="43" t="n"/>
+      <c r="AO39" s="49">
+        <f>IFERROR(AM39/AI39,"")</f>
+      </c>
+      <c r="AP39" s="43" t="n"/>
+      <c r="AQ39" s="51" t="n"/>
+      <c r="AR39" s="43" t="n"/>
+      <c r="AS39" s="43" t="inlineStr">
+        <is>
+          <t>Internal fixed + modular slots</t>
+        </is>
+      </c>
+      <c r="AT39" s="43" t="n">
+        <v>420</v>
+      </c>
+      <c r="AU39" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV39" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW39" s="43" t="inlineStr">
+        <is>
+          <t>B: APS600Wv3 / APS1200Wv2 / APS2000Wv2</t>
+        </is>
+      </c>
+      <c r="AX39" s="43" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="AY39" s="43" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="AZ39" s="43" t="n"/>
+      <c r="BA39" s="50">
+        <f>IF(MAX(AY39,AZ39)=0,"",ROUND(MAX(AY39,AZ39)*3.412,0))</f>
+        <v>552</v>
+      </c>
+      <c r="BB39" s="48" t="n">
+        <v>3200</v>
+      </c>
+      <c r="BC39" s="46" t="n">
+        <v>2380.8</v>
+      </c>
+      <c r="BD39" s="43" t="n">
+        <v>256</v>
+      </c>
+      <c r="BE39" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF39" s="43" t="inlineStr">
+        <is>
+          <t>Quad-core Cortex-A57 1.8GHz</t>
+        </is>
+      </c>
+      <c r="BG39" s="48" t="n">
+        <v>16384</v>
+      </c>
+      <c r="BH39" s="43" t="n">
+        <v>4093</v>
+      </c>
+      <c r="BI39" s="43" t="inlineStr">
+        <is>
+          <t>2K IPv4 / 2K IPv6</t>
+        </is>
+      </c>
+      <c r="BJ39" s="43" t="n"/>
+      <c r="BK39" s="43" t="inlineStr">
+        <is>
+          <t>Full L3 (static, RIP, OSPF, VRRP, PIM-SM/DM, PBR)</t>
+        </is>
+      </c>
+      <c r="BL39" s="43" t="inlineStr">
+        <is>
+          <t>Yes (NSF)</t>
+        </is>
+      </c>
+      <c r="BM39" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="BN39" s="43" t="inlineStr">
+        <is>
+          <t>Yes (exclusive with stacking)</t>
+        </is>
+      </c>
+      <c r="BO39" s="43" t="inlineStr">
+        <is>
+          <t>PTPv2 TC + Boundary/Grandmaster (SMPTE 2059-2, AES67, AES-R16)</t>
+        </is>
+      </c>
+      <c r="BP39" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BQ39" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BR39" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BS39" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="BT39" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="BU39" s="43" t="inlineStr">
+        <is>
+          <t>Front-to-back</t>
+        </is>
+      </c>
+      <c r="BV39" s="43" t="inlineStr">
+        <is>
+          <t>No (Quiet / Cool modes)</t>
+        </is>
+      </c>
+      <c r="BW39" s="43" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="BX39" s="48" t="n">
+        <v>390797</v>
+      </c>
+      <c r="BY39" s="43" t="inlineStr">
+        <is>
+          <t>ProSAFE Limited Lifetime HW; Lifetime NBD replacement</t>
+        </is>
+      </c>
+      <c r="BZ39" s="43" t="inlineStr">
+        <is>
+          <t>Sprint / Overdrive</t>
+        </is>
+      </c>
+      <c r="CA39" s="43" t="inlineStr">
+        <is>
+          <t>Yes (-TAANES)</t>
+        </is>
+      </c>
+      <c r="CB39" s="43" t="n"/>
+      <c r="CC39" s="43" t="n"/>
+      <c r="CD39" s="43" t="n"/>
+      <c r="CE39" s="43" t="n"/>
+      <c r="CF39" s="43" t="n"/>
+      <c r="CG39" s="43" t="n"/>
+      <c r="CH39" s="43" t="n"/>
+      <c r="CI39" s="43" t="n"/>
+      <c r="CJ39" s="43" t="n"/>
+      <c r="CK39" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="CL39" s="43" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="CM39" s="51" t="inlineStr">
+        <is>
+          <t>Packet buffer assumed 256 Mb (same as 16V4C/40X4C; datasheet table columns unclear). Modular slot = RPS only (no PoE)</t>
+        </is>
+      </c>
+      <c r="CN39" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO39" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
+      <c r="CP39" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" ht="46.25" customHeight="1" s="29">
+      <c r="A40" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B40" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>M4350</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR AV and IT</t>
+        </is>
+      </c>
+      <c r="E40" s="43" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F40" s="43" t="inlineStr">
+        <is>
+          <t>Access / Edge</t>
+        </is>
+      </c>
+      <c r="G40" s="43" t="inlineStr">
+        <is>
+          <t>AV UI; Engage; IT Web GUI; CLI; SNMP</t>
+        </is>
+      </c>
+      <c r="H40" s="43" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I40" s="44" t="n"/>
+      <c r="J40" s="45" t="n"/>
+      <c r="K40" s="45" t="n"/>
+      <c r="L40" s="43" t="inlineStr">
+        <is>
+          <t>1U rack</t>
+        </is>
+      </c>
+      <c r="M40" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="43" t="inlineStr">
+        <is>
+          <t>Full width</t>
+        </is>
+      </c>
+      <c r="O40" s="43" t="n">
+        <v>440</v>
+      </c>
+      <c r="P40" s="43" t="n">
+        <v>432</v>
+      </c>
+      <c r="Q40" s="43" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="R40" s="46" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="S40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" s="43" t="n">
+        <v>16</v>
+      </c>
+      <c r="U40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF40" s="47">
+        <f>SUM(S40:AE40)</f>
+        <v>20</v>
+      </c>
+      <c r="AG40" s="43" t="n"/>
+      <c r="AH40" s="43" t="inlineStr">
+        <is>
+          <t>8 of the 16 ports are Neutrik etherCON (front), 8 standard RJ45 (rear). Slot ships with APM414V: 4x SFP28 (17-20), 10G or 25G only. Other cards: APM414C 4x 10GBASE-T, APM414SD/LD opticalCON QUAD (MMF/SMF)</t>
+        </is>
+      </c>
+      <c r="AI40" s="43" t="n">
+        <v>16</v>
+      </c>
+      <c r="AJ40" s="43" t="inlineStr">
+        <is>
+          <t>802.3bt Ultra90 PoE++</t>
+        </is>
+      </c>
+      <c r="AK40" s="43" t="n">
+        <v>90</v>
+      </c>
+      <c r="AL40" s="48" t="n">
+        <v>530</v>
+      </c>
+      <c r="AM40" s="48" t="n">
+        <v>1130</v>
+      </c>
+      <c r="AN40" s="43" t="n">
+        <v>530</v>
+      </c>
+      <c r="AO40" s="49">
+        <f>IFERROR(AM40/AI40,"")</f>
+        <v>70.625</v>
+      </c>
+      <c r="AP40" s="43" t="n"/>
+      <c r="AQ40" s="51" t="n"/>
+      <c r="AR40" s="43" t="n"/>
+      <c r="AS40" s="43" t="inlineStr">
+        <is>
+          <t>2x internal 800W (powerCON), 1+1</t>
+        </is>
+      </c>
+      <c r="AT40" s="43" t="n">
+        <v>800</v>
+      </c>
+      <c r="AU40" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV40" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW40" s="43" t="inlineStr">
+        <is>
+          <t>None (2 internal)</t>
+        </is>
+      </c>
+      <c r="AX40" s="43" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="AY40" s="43" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="AZ40" s="43" t="n">
+        <v>1359.8</v>
+      </c>
+      <c r="BA40" s="50">
+        <f>IF(MAX(AY40,AZ40)=0,"",ROUND(MAX(AY40,AZ40)*3.412,0))</f>
+        <v>4640</v>
+      </c>
+      <c r="BB40" s="48" t="n">
+        <v>280</v>
+      </c>
+      <c r="BC40" s="46" t="n">
+        <v>208.32</v>
+      </c>
+      <c r="BD40" s="43" t="n">
+        <v>32</v>
+      </c>
+      <c r="BE40" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF40" s="43" t="inlineStr">
+        <is>
+          <t>Quad-core Cortex-A57 1.8GHz</t>
+        </is>
+      </c>
+      <c r="BG40" s="48" t="n">
+        <v>16384</v>
+      </c>
+      <c r="BH40" s="43" t="n">
+        <v>4093</v>
+      </c>
+      <c r="BI40" s="43" t="inlineStr">
+        <is>
+          <t>2K IPv4 / 2K IPv6</t>
+        </is>
+      </c>
+      <c r="BJ40" s="43" t="n"/>
+      <c r="BK40" s="43" t="inlineStr">
+        <is>
+          <t>Full L3 (static, RIP, OSPF, VRRP, PIM-SM/DM, PBR)</t>
+        </is>
+      </c>
+      <c r="BL40" s="43" t="inlineStr">
+        <is>
+          <t>Yes (NSF)</t>
+        </is>
+      </c>
+      <c r="BM40" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="BN40" s="43" t="inlineStr">
+        <is>
+          <t>Yes (exclusive with stacking)</t>
+        </is>
+      </c>
+      <c r="BO40" s="43" t="inlineStr">
+        <is>
+          <t>PTPv2 TC + Boundary/Grandmaster (SMPTE 2059-2, AES67, AES-R16)</t>
+        </is>
+      </c>
+      <c r="BP40" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BQ40" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BR40" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BS40" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="BT40" s="43" t="n">
+        <v>45</v>
+      </c>
+      <c r="BU40" s="43" t="inlineStr">
+        <is>
+          <t>Front-to-back</t>
+        </is>
+      </c>
+      <c r="BV40" s="43" t="inlineStr">
+        <is>
+          <t>No (Quiet / Cool modes)</t>
+        </is>
+      </c>
+      <c r="BW40" s="43" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="BX40" s="48" t="n">
+        <v>355650</v>
+      </c>
+      <c r="BY40" s="43" t="inlineStr">
+        <is>
+          <t>ProSAFE Limited Lifetime HW; Lifetime NBD replacement</t>
+        </is>
+      </c>
+      <c r="BZ40" s="43" t="inlineStr">
+        <is>
+          <t>Sprint / Overdrive</t>
+        </is>
+      </c>
+      <c r="CA40" s="43" t="inlineStr">
+        <is>
+          <t>Yes (-TAANES)</t>
+        </is>
+      </c>
+      <c r="CB40" s="43" t="n"/>
+      <c r="CC40" s="43" t="n"/>
+      <c r="CD40" s="43" t="n"/>
+      <c r="CE40" s="43" t="n"/>
+      <c r="CF40" s="43" t="n"/>
+      <c r="CG40" s="43" t="n"/>
+      <c r="CH40" s="43" t="n"/>
+      <c r="CI40" s="43" t="n"/>
+      <c r="CJ40" s="43" t="n"/>
+      <c r="CK40" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="CL40" s="43" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="CM40" s="51" t="inlineStr">
+        <is>
+          <t>Ports modelled with the shipping APM414V card (4x SFP28). Packet buffer and RAM assumed as 8M2V. powerCON inputs, C14 adapters included</t>
+        </is>
+      </c>
+      <c r="CN40" s="51" t="inlineStr">
+        <is>
+          <t>Sprint, Overdrive, Fastlane</t>
+        </is>
+      </c>
+      <c r="CO40" s="51" t="inlineStr">
+        <is>
+          <t>Sprint 3 yr</t>
+        </is>
+      </c>
+      <c r="CP40" s="51" t="n">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:CO1"/>
-    <mergeCell ref="A2:CO2"/>
+    <mergeCell ref="A1:CP1"/>
+    <mergeCell ref="A2:CP2"/>
   </mergeCells>
   <dataValidations count="8">
     <dataValidation sqref="E5:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
@@ -18352,7 +19161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G149"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -23198,6 +24007,270 @@
         </is>
       </c>
       <c r="G149" s="43" t="n"/>
+    </row>
+    <row r="150" ht="15" customHeight="1" s="29">
+      <c r="A150" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B150" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C150" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316-100NES</t>
+        </is>
+      </c>
+      <c r="D150" s="43" t="inlineStr">
+        <is>
+          <t>Americas / Europe</t>
+        </is>
+      </c>
+      <c r="E150" s="43" t="inlineStr">
+        <is>
+          <t>NA, UK, EU cords</t>
+        </is>
+      </c>
+      <c r="F150" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G150" s="43" t="n"/>
+    </row>
+    <row r="151" ht="15" customHeight="1" s="29">
+      <c r="A151" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B151" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C151" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316-TAANES</t>
+        </is>
+      </c>
+      <c r="D151" s="43" t="inlineStr">
+        <is>
+          <t>Americas (TAA)</t>
+        </is>
+      </c>
+      <c r="E151" s="43" t="inlineStr">
+        <is>
+          <t>NA, UK, EU cords</t>
+        </is>
+      </c>
+      <c r="F151" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G151" s="43" t="n"/>
+    </row>
+    <row r="152" ht="15" customHeight="1" s="29">
+      <c r="A152" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B152" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C152" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316-100AJS</t>
+        </is>
+      </c>
+      <c r="D152" s="43" t="inlineStr">
+        <is>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="E152" s="43" t="inlineStr">
+        <is>
+          <t>JP, AU cords</t>
+        </is>
+      </c>
+      <c r="F152" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G152" s="43" t="n"/>
+    </row>
+    <row r="153" ht="15" customHeight="1" s="29">
+      <c r="A153" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B153" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C153" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316-100PRS</t>
+        </is>
+      </c>
+      <c r="D153" s="43" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E153" s="43" t="inlineStr">
+        <is>
+          <t>CN cord</t>
+        </is>
+      </c>
+      <c r="F153" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G153" s="43" t="n"/>
+    </row>
+    <row r="154" ht="15" customHeight="1" s="29">
+      <c r="A154" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B154" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C154" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320-100NES</t>
+        </is>
+      </c>
+      <c r="D154" s="43" t="inlineStr">
+        <is>
+          <t>Americas / Europe</t>
+        </is>
+      </c>
+      <c r="E154" s="43" t="inlineStr">
+        <is>
+          <t>NA, UK, EU cords</t>
+        </is>
+      </c>
+      <c r="F154" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G154" s="43" t="n"/>
+    </row>
+    <row r="155" ht="15" customHeight="1" s="29">
+      <c r="A155" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B155" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C155" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320-TAANES</t>
+        </is>
+      </c>
+      <c r="D155" s="43" t="inlineStr">
+        <is>
+          <t>Americas (TAA)</t>
+        </is>
+      </c>
+      <c r="E155" s="43" t="inlineStr">
+        <is>
+          <t>NA, UK, EU cords</t>
+        </is>
+      </c>
+      <c r="F155" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G155" s="43" t="n"/>
+    </row>
+    <row r="156" ht="15" customHeight="1" s="29">
+      <c r="A156" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B156" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C156" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320-100AJS</t>
+        </is>
+      </c>
+      <c r="D156" s="43" t="inlineStr">
+        <is>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="E156" s="43" t="inlineStr">
+        <is>
+          <t>JP, AU cords</t>
+        </is>
+      </c>
+      <c r="F156" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G156" s="43" t="n"/>
+    </row>
+    <row r="157" ht="15" customHeight="1" s="29">
+      <c r="A157" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B157" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C157" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320-100PRS</t>
+        </is>
+      </c>
+      <c r="D157" s="43" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E157" s="43" t="inlineStr">
+        <is>
+          <t>CN cord</t>
+        </is>
+      </c>
+      <c r="F157" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G157" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -23219,7 +24292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q127"/>
+  <dimension ref="A1:Q131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="28" min="1" max="1"/>
@@ -30191,6 +31264,234 @@
       </c>
       <c r="Q127" s="43" t="n"/>
     </row>
+    <row r="128" ht="23.85" customHeight="1" s="29">
+      <c r="A128" s="43" t="inlineStr">
+        <is>
+          <t>APM414V-10000S</t>
+        </is>
+      </c>
+      <c r="B128" s="43" t="inlineStr">
+        <is>
+          <t>APM414V</t>
+        </is>
+      </c>
+      <c r="C128" s="43" t="inlineStr">
+        <is>
+          <t>Interface Card</t>
+        </is>
+      </c>
+      <c r="D128" s="51" t="inlineStr">
+        <is>
+          <t>APM414V card: 4x standard SFP28 (10G/25G), ships pre-installed in the M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="E128" s="43" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="F128" s="43" t="n"/>
+      <c r="G128" s="43" t="n"/>
+      <c r="H128" s="43" t="inlineStr">
+        <is>
+          <t>SFP28</t>
+        </is>
+      </c>
+      <c r="I128" s="43" t="n"/>
+      <c r="J128" s="43" t="n"/>
+      <c r="K128" s="43" t="n"/>
+      <c r="L128" s="43" t="n"/>
+      <c r="M128" s="43" t="n"/>
+      <c r="N128" s="43" t="n"/>
+      <c r="O128" s="43" t="inlineStr">
+        <is>
+          <t>Lifetime</t>
+        </is>
+      </c>
+      <c r="P128" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="Q128" s="43" t="inlineStr">
+        <is>
+          <t>Included with MSM4320. AOC recommended for 25G (passive DAC can take 15-70 s to link)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="23.85" customHeight="1" s="29">
+      <c r="A129" s="43" t="inlineStr">
+        <is>
+          <t>APM414C-10000S</t>
+        </is>
+      </c>
+      <c r="B129" s="43" t="inlineStr">
+        <is>
+          <t>APM414C</t>
+        </is>
+      </c>
+      <c r="C129" s="43" t="inlineStr">
+        <is>
+          <t>Interface Card</t>
+        </is>
+      </c>
+      <c r="D129" s="51" t="inlineStr">
+        <is>
+          <t>APM414C card: 4x 10GBASE-T RJ45 (1G/10G only)</t>
+        </is>
+      </c>
+      <c r="E129" s="43" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="F129" s="43" t="n"/>
+      <c r="G129" s="43" t="n"/>
+      <c r="H129" s="43" t="inlineStr">
+        <is>
+          <t>RJ45</t>
+        </is>
+      </c>
+      <c r="I129" s="43" t="n"/>
+      <c r="J129" s="43" t="n"/>
+      <c r="K129" s="43" t="n"/>
+      <c r="L129" s="43" t="n"/>
+      <c r="M129" s="43" t="n"/>
+      <c r="N129" s="43" t="n"/>
+      <c r="O129" s="43" t="inlineStr">
+        <is>
+          <t>Lifetime</t>
+        </is>
+      </c>
+      <c r="P129" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="Q129" s="43" t="inlineStr">
+        <is>
+          <t>Optional for MSM4320. No 100M/2.5G/5G</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="23.85" customHeight="1" s="29">
+      <c r="A130" s="43" t="inlineStr">
+        <is>
+          <t>APM414SD-10000S</t>
+        </is>
+      </c>
+      <c r="B130" s="43" t="inlineStr">
+        <is>
+          <t>APM414SD</t>
+        </is>
+      </c>
+      <c r="C130" s="43" t="inlineStr">
+        <is>
+          <t>Interface Card</t>
+        </is>
+      </c>
+      <c r="D130" s="51" t="inlineStr">
+        <is>
+          <t>APM414SD card: 2x Neutrik opticalCON QUAD, 4 internal SFP28 cages for 10G/25G multimode transceivers</t>
+        </is>
+      </c>
+      <c r="E130" s="43" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="F130" s="43" t="n"/>
+      <c r="G130" s="43" t="inlineStr">
+        <is>
+          <t>MMF</t>
+        </is>
+      </c>
+      <c r="H130" s="43" t="inlineStr">
+        <is>
+          <t>opticalCON QUAD</t>
+        </is>
+      </c>
+      <c r="I130" s="43" t="n"/>
+      <c r="J130" s="43" t="n"/>
+      <c r="K130" s="43" t="n"/>
+      <c r="L130" s="43" t="n"/>
+      <c r="M130" s="43" t="n"/>
+      <c r="N130" s="43" t="n"/>
+      <c r="O130" s="43" t="inlineStr">
+        <is>
+          <t>Lifetime</t>
+        </is>
+      </c>
+      <c r="P130" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="Q130" s="43" t="inlineStr">
+        <is>
+          <t>Optional for MSM4320. Includes 4 MMF patch cords to the opticalCON connectors; transceivers ordered separately</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="23.85" customHeight="1" s="29">
+      <c r="A131" s="43" t="inlineStr">
+        <is>
+          <t>APM414LD-10000S</t>
+        </is>
+      </c>
+      <c r="B131" s="43" t="inlineStr">
+        <is>
+          <t>APM414LD</t>
+        </is>
+      </c>
+      <c r="C131" s="43" t="inlineStr">
+        <is>
+          <t>Interface Card</t>
+        </is>
+      </c>
+      <c r="D131" s="51" t="inlineStr">
+        <is>
+          <t>APM414LD card: 2x Neutrik opticalCON QUAD, 4 internal SFP28 cages for 10G/25G single mode transceivers</t>
+        </is>
+      </c>
+      <c r="E131" s="43" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="F131" s="43" t="n"/>
+      <c r="G131" s="43" t="inlineStr">
+        <is>
+          <t>SMF</t>
+        </is>
+      </c>
+      <c r="H131" s="43" t="inlineStr">
+        <is>
+          <t>opticalCON QUAD</t>
+        </is>
+      </c>
+      <c r="I131" s="43" t="n"/>
+      <c r="J131" s="43" t="n"/>
+      <c r="K131" s="43" t="n"/>
+      <c r="L131" s="43" t="n"/>
+      <c r="M131" s="43" t="n"/>
+      <c r="N131" s="43" t="n"/>
+      <c r="O131" s="43" t="inlineStr">
+        <is>
+          <t>Lifetime</t>
+        </is>
+      </c>
+      <c r="P131" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+      <c r="Q131" s="43" t="inlineStr">
+        <is>
+          <t>Optional for MSM4320. Includes 4 SMF patch cords to the opticalCON connectors; transceivers ordered separately</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -30198,7 +31499,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C5:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>Lists!$H$5:$H$17</formula1>
+      <formula1>Lists!$H$5:$H$18</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -30217,7 +31518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G172"/>
+  <dimension ref="A1:G176"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="28" min="1" max="1"/>
@@ -35845,7 +37146,7 @@
         </is>
       </c>
     </row>
-    <row r="172">
+    <row r="172" s="29">
       <c r="A172" s="43" t="inlineStr">
         <is>
           <t>Product</t>
@@ -35875,6 +37176,146 @@
       <c r="G172" s="43" t="inlineStr">
         <is>
           <t>Used only when no 10G port is free: 1G SX module on both ends. Confirm the PR460X SFP+ port accepts 1G modules</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B173" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="C173" s="43" t="inlineStr">
+        <is>
+          <t>Interface card slot</t>
+        </is>
+      </c>
+      <c r="D173" s="43" t="inlineStr">
+        <is>
+          <t>APM414V</t>
+        </is>
+      </c>
+      <c r="E173" s="43" t="inlineStr">
+        <is>
+          <t>Interface card (included)</t>
+        </is>
+      </c>
+      <c r="F173" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G173" s="43" t="inlineStr">
+        <is>
+          <t>Ships installed; 4x SFP28 10G/25G</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B174" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="C174" s="43" t="inlineStr">
+        <is>
+          <t>Interface card slot</t>
+        </is>
+      </c>
+      <c r="D174" s="43" t="inlineStr">
+        <is>
+          <t>APM414C</t>
+        </is>
+      </c>
+      <c r="E174" s="43" t="inlineStr">
+        <is>
+          <t>Optional interface card</t>
+        </is>
+      </c>
+      <c r="F174" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G174" s="43" t="inlineStr">
+        <is>
+          <t>Replaces APM414V: 4x 10GBASE-T</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B175" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="C175" s="43" t="inlineStr">
+        <is>
+          <t>Interface card slot</t>
+        </is>
+      </c>
+      <c r="D175" s="43" t="inlineStr">
+        <is>
+          <t>APM414SD</t>
+        </is>
+      </c>
+      <c r="E175" s="43" t="inlineStr">
+        <is>
+          <t>Optional interface card</t>
+        </is>
+      </c>
+      <c r="F175" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G175" s="43" t="inlineStr">
+        <is>
+          <t>Replaces APM414V: opticalCON QUAD, multimode optics in internal cages</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="43" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B176" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="C176" s="43" t="inlineStr">
+        <is>
+          <t>Interface card slot</t>
+        </is>
+      </c>
+      <c r="D176" s="43" t="inlineStr">
+        <is>
+          <t>APM414LD</t>
+        </is>
+      </c>
+      <c r="E176" s="43" t="inlineStr">
+        <is>
+          <t>Optional interface card</t>
+        </is>
+      </c>
+      <c r="F176" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G176" s="43" t="inlineStr">
+        <is>
+          <t>Replaces APM414V: opticalCON QUAD, single mode optics in internal cages</t>
         </is>
       </c>
     </row>
@@ -35904,7 +37345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -40850,6 +42291,361 @@
       <c r="L107" s="43" t="inlineStr">
         <is>
           <t>Both PSUs ship with the switch; no PoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1" s="29">
+      <c r="A108" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B108" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C108" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D108" s="43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E108" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="43" t="inlineStr">
+        <is>
+          <t>110-240 VAC</t>
+        </is>
+      </c>
+      <c r="G108" s="48" t="n"/>
+      <c r="H108" s="48" t="n"/>
+      <c r="I108" s="48" t="n"/>
+      <c r="J108" s="50">
+        <f>IF(COUNT(H108,I108)=0,"",MIN(H108,I108))</f>
+      </c>
+      <c r="K108" s="43" t="inlineStr">
+        <is>
+          <t>Base (no module)</t>
+        </is>
+      </c>
+      <c r="L108" s="43" t="inlineStr">
+        <is>
+          <t>Base budget, no redundancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="29">
+      <c r="A109" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B109" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C109" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D109" s="43" t="inlineStr">
+        <is>
+          <t>APS600Wv3</t>
+        </is>
+      </c>
+      <c r="E109" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="43" t="inlineStr">
+        <is>
+          <t>110-240 VAC</t>
+        </is>
+      </c>
+      <c r="G109" s="48" t="n"/>
+      <c r="H109" s="48" t="n"/>
+      <c r="I109" s="48" t="n"/>
+      <c r="J109" s="50">
+        <f>IF(COUNT(H109,I109)=0,"",MIN(H109,I109))</f>
+      </c>
+      <c r="K109" s="43" t="inlineStr">
+        <is>
+          <t>1x APS600Wv3</t>
+        </is>
+      </c>
+      <c r="L109" s="43" t="n"/>
+    </row>
+    <row r="110" ht="15" customHeight="1" s="29">
+      <c r="A110" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B110" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C110" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D110" s="43" t="inlineStr">
+        <is>
+          <t>APS1200Wv2</t>
+        </is>
+      </c>
+      <c r="E110" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="43" t="inlineStr">
+        <is>
+          <t>110 VAC</t>
+        </is>
+      </c>
+      <c r="G110" s="48" t="n"/>
+      <c r="H110" s="48" t="n"/>
+      <c r="I110" s="48" t="n"/>
+      <c r="J110" s="50">
+        <f>IF(COUNT(H110,I110)=0,"",MIN(H110,I110))</f>
+      </c>
+      <c r="K110" s="43" t="inlineStr">
+        <is>
+          <t>1x APS1200Wv2 @110V</t>
+        </is>
+      </c>
+      <c r="L110" s="43" t="n"/>
+    </row>
+    <row r="111" ht="15" customHeight="1" s="29">
+      <c r="A111" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B111" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C111" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D111" s="43" t="inlineStr">
+        <is>
+          <t>APS1200Wv2</t>
+        </is>
+      </c>
+      <c r="E111" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="43" t="inlineStr">
+        <is>
+          <t>220 VAC</t>
+        </is>
+      </c>
+      <c r="G111" s="48" t="n"/>
+      <c r="H111" s="48" t="n"/>
+      <c r="I111" s="48" t="n"/>
+      <c r="J111" s="50">
+        <f>IF(COUNT(H111,I111)=0,"",MIN(H111,I111))</f>
+      </c>
+      <c r="K111" s="43" t="inlineStr">
+        <is>
+          <t>1x APS1200Wv2 @220V</t>
+        </is>
+      </c>
+      <c r="L111" s="43" t="n"/>
+    </row>
+    <row r="112" ht="15" customHeight="1" s="29">
+      <c r="A112" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B112" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C112" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D112" s="43" t="inlineStr">
+        <is>
+          <t>APS2000Wv2</t>
+        </is>
+      </c>
+      <c r="E112" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="43" t="inlineStr">
+        <is>
+          <t>110 VAC</t>
+        </is>
+      </c>
+      <c r="G112" s="48" t="n"/>
+      <c r="H112" s="48" t="n"/>
+      <c r="I112" s="48" t="n"/>
+      <c r="J112" s="50">
+        <f>IF(COUNT(H112,I112)=0,"",MIN(H112,I112))</f>
+      </c>
+      <c r="K112" s="43" t="inlineStr">
+        <is>
+          <t>1x APS2000Wv2 @110V</t>
+        </is>
+      </c>
+      <c r="L112" s="43" t="n"/>
+    </row>
+    <row r="113" ht="15" customHeight="1" s="29">
+      <c r="A113" s="43" t="inlineStr">
+        <is>
+          <t>CSM4316</t>
+        </is>
+      </c>
+      <c r="B113" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16C</t>
+        </is>
+      </c>
+      <c r="C113" s="43" t="inlineStr">
+        <is>
+          <t>420W internal</t>
+        </is>
+      </c>
+      <c r="D113" s="43" t="inlineStr">
+        <is>
+          <t>APS2000Wv2</t>
+        </is>
+      </c>
+      <c r="E113" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="43" t="inlineStr">
+        <is>
+          <t>220 VAC</t>
+        </is>
+      </c>
+      <c r="G113" s="48" t="n"/>
+      <c r="H113" s="48" t="n"/>
+      <c r="I113" s="48" t="n"/>
+      <c r="J113" s="50">
+        <f>IF(COUNT(H113,I113)=0,"",MIN(H113,I113))</f>
+      </c>
+      <c r="K113" s="43" t="inlineStr">
+        <is>
+          <t>1x APS2000Wv2 @220V</t>
+        </is>
+      </c>
+      <c r="L113" s="43" t="n"/>
+    </row>
+    <row r="114" ht="15" customHeight="1" s="29">
+      <c r="A114" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B114" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C114" s="43" t="inlineStr">
+        <is>
+          <t>2x 800W internal</t>
+        </is>
+      </c>
+      <c r="D114" s="43" t="inlineStr">
+        <is>
+          <t>(internal PSUs)</t>
+        </is>
+      </c>
+      <c r="E114" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="43" t="inlineStr">
+        <is>
+          <t>110-240 VAC</t>
+        </is>
+      </c>
+      <c r="G114" s="48" t="n">
+        <v>530</v>
+      </c>
+      <c r="H114" s="48" t="n"/>
+      <c r="I114" s="48" t="n"/>
+      <c r="J114" s="50">
+        <f>IF(COUNT(H114,I114)=0,"",MIN(H114,I114))</f>
+      </c>
+      <c r="K114" s="43" t="inlineStr">
+        <is>
+          <t>1 of 2 PSUs powered</t>
+        </is>
+      </c>
+      <c r="L114" s="43" t="inlineStr">
+        <is>
+          <t>No redundancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="15" customHeight="1" s="29">
+      <c r="A115" s="43" t="inlineStr">
+        <is>
+          <t>MSM4320</t>
+        </is>
+      </c>
+      <c r="B115" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C115" s="43" t="inlineStr">
+        <is>
+          <t>2x 800W internal</t>
+        </is>
+      </c>
+      <c r="D115" s="43" t="inlineStr">
+        <is>
+          <t>(internal PSUs)</t>
+        </is>
+      </c>
+      <c r="E115" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F115" s="43" t="inlineStr">
+        <is>
+          <t>110-240 VAC</t>
+        </is>
+      </c>
+      <c r="G115" s="48" t="n">
+        <v>1130</v>
+      </c>
+      <c r="H115" s="48" t="n"/>
+      <c r="I115" s="48" t="n">
+        <v>530</v>
+      </c>
+      <c r="J115" s="50">
+        <f>IF(COUNT(H115,I115)=0,"",MIN(H115,I115))</f>
+        <v>530</v>
+      </c>
+      <c r="K115" s="43" t="inlineStr">
+        <is>
+          <t>2 of 2 PSUs powered</t>
+        </is>
+      </c>
+      <c r="L115" s="43" t="inlineStr">
+        <is>
+          <t>1+1: 530W protected</t>
         </is>
       </c>
     </row>
@@ -40873,7 +42669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="28" min="1" max="1"/>
@@ -41535,6 +43331,70 @@
       <c r="F23" s="43" t="inlineStr">
         <is>
           <t>ProAV Design team</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="23.85" customHeight="1" s="29">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>M4350-16M4V</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>Ports</t>
+        </is>
+      </c>
+      <c r="D24" s="51" t="inlineStr">
+        <is>
+          <t>One interface card slot: APM414V (4x SFP28, installed), APM414C (4x 10GBASE-T), APM414SD/LD (opticalCON QUAD, MMF/SMF). One card at a time.</t>
+        </is>
+      </c>
+      <c r="E24" s="51" t="inlineStr">
+        <is>
+          <t>Uplink media follows the card; opticalCON cards need SFP28/SFP+ transceivers in the internal cages and Neutrik opticalCON field cables.</t>
+        </is>
+      </c>
+      <c r="F24" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="23.85" customHeight="1" s="29">
+      <c r="A25" s="43" t="inlineStr">
+        <is>
+          <t>R21</t>
+        </is>
+      </c>
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>M4350 (all)</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="inlineStr">
+        <is>
+          <t>AVB</t>
+        </is>
+      </c>
+      <c r="D25" s="51" t="inlineStr">
+        <is>
+          <t>In a LAG only one physical link carries AVB payload; the other links are backup.</t>
+        </is>
+      </c>
+      <c r="E25" s="51" t="inlineStr">
+        <is>
+          <t>AVB bandwidth through a LAG is one link, not the LAG total.</t>
+        </is>
+      </c>
+      <c r="F25" s="43" t="inlineStr">
+        <is>
+          <t>M4350 datasheet DS-M4350-03Jul26 (M4350_Datasheet.pdf)</t>
         </is>
       </c>
     </row>
@@ -41909,7 +43769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="28" min="1" max="1"/>
@@ -42468,7 +44328,7 @@
       </c>
       <c r="J17" s="43" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" s="29">
       <c r="A18" s="43" t="inlineStr">
         <is>
           <t>EP-MILAN</t>
@@ -42507,6 +44367,48 @@
       <c r="J18" s="43" t="inlineStr">
         <is>
           <t>AVB</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>EP-2110-AUDIO</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>ST 2110-30 / AES67 audio device</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="43" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="F19" s="45" t="n">
+        <v>13</v>
+      </c>
+      <c r="G19" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="43" t="n"/>
+      <c r="I19" s="43" t="inlineStr">
+        <is>
+          <t>PTP (SMPTE 2059-2 / AES67) via boundary clock switches. Clear Timing if your design uses transparent clock only</t>
+        </is>
+      </c>
+      <c r="J19" s="43" t="inlineStr">
+        <is>
+          <t>PTP-BC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Compare designs on cost with a published cost index
- Engine compares complete designs on cost: switches, PSU modules, optics
  and cables, plus a per-switch overhead; unpriced items are estimated from
  parts of the same kind; new 'cheapest links' uplink strategy
- Public catalog carries a relative Cost_Index (no prices or sources);
  real prices are kept privately and published with tools/publish_costs.py
- Copper RJ45 modules keep a penalty, preferred uplink speed is near-
  mandatory, core ports weigh more in the fastest-uplinks strategy
- Diagram labels third-party placeholders; validation scenarios V40-V41,
  summary with relative cost, docs and reports
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1058,9 +1058,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CP40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProducts" displayName="tblProducts" ref="A4:CQ40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:CM38"/>
-  <tableColumns count="94">
+  <tableColumns count="95">
     <tableColumn id="1" name="Product_ID"/>
     <tableColumn id="2" name="Model_Name"/>
     <tableColumn id="3" name="Family"/>
@@ -1069,7 +1069,7 @@
     <tableColumn id="6" name="Role"/>
     <tableColumn id="7" name="Management"/>
     <tableColumn id="8" name="Lifecycle_Status"/>
-    <tableColumn id="9" name="List_Price_USD"/>
+    <tableColumn id="9" name="Cost_Index"/>
     <tableColumn id="10" name="Lead_Time_Wks"/>
     <tableColumn id="11" name="EOS_Date"/>
     <tableColumn id="12" name="Form_Factor"/>
@@ -1155,12 +1155,13 @@
     <tableColumn id="92" name="Support_Tiers"/>
     <tableColumn id="93" name="Included_Support"/>
     <tableColumn id="94" name="Neutrik_etherCON_Ports"/>
+    <tableColumn id="95" name="Cost_Note"/>
   </tableColumns>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F117" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F113"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Sheet"/>
@@ -1200,9 +1201,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:Q131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:S131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:Q127"/>
-  <tableColumns count="17">
+  <tableColumns count="19">
     <tableColumn id="1" name="Orderable_SKU"/>
     <tableColumn id="2" name="Base_Model"/>
     <tableColumn id="3" name="Category"/>
@@ -1220,6 +1221,8 @@
     <tableColumn id="15" name="Warranty"/>
     <tableColumn id="16" name="Source"/>
     <tableColumn id="17" name="Notes"/>
+    <tableColumn id="18" name="Cost_Index"/>
+    <tableColumn id="19" name="Cost_Note"/>
   </tableColumns>
 </table>
 </file>
@@ -1311,7 +1314,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Key"/>
@@ -2696,7 +2699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="28" min="1" max="1"/>
@@ -2743,7 +2746,7 @@
       </c>
       <c r="B5" s="43" t="inlineStr">
         <is>
-          <t>2026.10.01c</t>
+          <t>2026.10.01d</t>
         </is>
       </c>
       <c r="C5" s="43" t="inlineStr">
@@ -2840,25 +2843,29 @@
     <row r="11" ht="15" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
         <is>
-          <t>Default_Spare_Pct</t>
+          <t>Per_Switch_Overhead</t>
         </is>
       </c>
       <c r="B11" s="43" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="n"/>
+          <t>3210</t>
+        </is>
+      </c>
+      <c r="C11" s="51" t="inlineStr">
+        <is>
+          <t>Added to every switch when comparing designs, in Cost_Index units: rack space, power, patching and setup. Higher values favor fewer, larger switches</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>Default_PoE_Headroom_Pct</t>
+          <t>Default_Spare_Pct</t>
         </is>
       </c>
       <c r="B12" s="43" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C12" s="43" t="n"/>
@@ -2866,134 +2873,147 @@
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
         <is>
-          <t>Default_Oversubscription</t>
+          <t>Default_PoE_Headroom_Pct</t>
         </is>
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>1 = line-rate</t>
-        </is>
-      </c>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
         <is>
-          <t>Max_LAG_Members</t>
+          <t>Default_Oversubscription</t>
         </is>
       </c>
       <c r="B14" s="43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C14" s="43" t="inlineStr">
         <is>
-          <t>Max uplinks per switch</t>
+          <t>1 = line-rate</t>
         </is>
       </c>
     </row>
     <row r="15" ht="23.85" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
         <is>
-          <t>Min_Uplink_Gbps</t>
+          <t>Max_LAG_Members</t>
         </is>
       </c>
       <c r="B15" s="43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C15" s="43" t="inlineStr">
         <is>
-          <t>Slowest uplink speed to the core. 1 allows 1G uplinks when the bandwidth fits (for example audio on stream bandwidth); raise to 10 to force 10G uplinks everywhere</t>
+          <t>Max uplinks per switch</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
         <is>
-          <t>Stream_Uplink_Headroom_Pct</t>
+          <t>Min_Uplink_Gbps</t>
         </is>
       </c>
       <c r="B16" s="43" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>Stream bandwidth basis only: uplinks must carry the stream total plus this margin, because stream rates are typical, not peak. Line-rate needs no margin</t>
+          <t>Slowest uplink speed to the core. 1 allows 1G uplinks when the bandwidth fits (for example audio on stream bandwidth); raise to 10 to force 10G uplinks everywhere</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
         <is>
-          <t>Uplink_LAG_Sizes</t>
+          <t>Stream_Uplink_Headroom_Pct</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
         <is>
-          <t>1,2,4,8</t>
-        </is>
-      </c>
-      <c r="C17" s="51" t="inlineStr">
-        <is>
-          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Stream bandwidth basis only: uplinks must carry the stream total plus this margin, because stream rates are typical, not peak. Line-rate needs no margin</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
         <is>
-          <t>In_Rack_Max_m</t>
+          <t>Uplink_LAG_Sizes</t>
         </is>
       </c>
       <c r="B18" s="43" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>MDF links at or below this use DAC/AOC</t>
+          <t>1,2,4,8</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="inlineStr">
+        <is>
+          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
         <is>
-          <t>Copper_10G_Max_m</t>
+          <t>In_Rack_Max_m</t>
         </is>
       </c>
       <c r="B19" s="43" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C19" s="43" t="inlineStr">
         <is>
-          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+          <t>MDF links at or below this use DAC/AOC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
         <is>
+          <t>Copper_10G_Max_m</t>
+        </is>
+      </c>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
           <t>Endpoint_Speeds_Gbps</t>
         </is>
       </c>
-      <c r="B20" s="43" t="inlineStr">
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>1,2.5,5,10,25,50,100</t>
         </is>
       </c>
-      <c r="C20" s="43" t="inlineStr">
+      <c r="C21" s="43" t="inlineStr">
         <is>
           <t>Speeds offered in the endpoint library</t>
         </is>
@@ -3019,7 +3039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="28" min="1" max="1"/>
@@ -3308,7 +3328,7 @@
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>List_Price_USD</t>
+          <t>Cost_Index</t>
         </is>
       </c>
       <c r="C13" s="43" t="inlineStr">
@@ -3316,11 +3336,7 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="D13" s="43" t="n"/>
       <c r="E13" s="43" t="inlineStr">
         <is>
           <t>Number</t>
@@ -3328,7 +3344,7 @@
       </c>
       <c r="F13" s="43" t="inlineStr">
         <is>
-          <t>TO FILL from price book</t>
+          <t>Relative cost used to compare designs. Not a price: real prices are kept internally</t>
         </is>
       </c>
     </row>
@@ -6417,6 +6433,90 @@
       <c r="F117" s="51" t="inlineStr">
         <is>
           <t>Locking Neutrik etherCON RJ45 ports (front). 0 = standard RJ45 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="43" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="B118" s="51" t="inlineStr">
+        <is>
+          <t>Cost_Note</t>
+        </is>
+      </c>
+      <c r="C118" s="43" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D118" s="43" t="n"/>
+      <c r="E118" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F118" s="51" t="inlineStr">
+        <is>
+          <t>Notes on the cost index (no sources published)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="43" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B119" s="51" t="inlineStr">
+        <is>
+          <t>Cost_Index</t>
+        </is>
+      </c>
+      <c r="C119" s="43" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D119" s="43" t="n"/>
+      <c r="E119" s="43" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="F119" s="51" t="inlineStr">
+        <is>
+          <t>Relative cost used to compare designs. Not a price: real prices are kept internally</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="43" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B120" s="51" t="inlineStr">
+        <is>
+          <t>Cost_Note</t>
+        </is>
+      </c>
+      <c r="C120" s="43" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D120" s="43" t="n"/>
+      <c r="E120" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F120" s="51" t="inlineStr">
+        <is>
+          <t>Notes on the cost index (no sources published)</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:CP40"/>
+  <dimension ref="A1:CQ40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="28" min="1" max="1"/>
@@ -7361,6 +7461,7 @@
     <col width="26" customWidth="1" style="29" min="92" max="92"/>
     <col width="26" customWidth="1" style="29" min="93" max="93"/>
     <col width="14" customWidth="1" style="29" min="94" max="94"/>
+    <col width="40" customWidth="1" style="29" min="95" max="95"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -7569,7 +7670,7 @@
       </c>
       <c r="I4" s="42" t="inlineStr">
         <is>
-          <t>List_Price_USD</t>
+          <t>Cost_Index</t>
         </is>
       </c>
       <c r="J4" s="42" t="inlineStr">
@@ -7995,6 +8096,11 @@
       <c r="CP4" s="42" t="inlineStr">
         <is>
           <t>Neutrik_etherCON_Ports</t>
+        </is>
+      </c>
+      <c r="CQ4" s="42" t="inlineStr">
+        <is>
+          <t>Cost_Note</t>
         </is>
       </c>
     </row>
@@ -8039,7 +8145,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I5" s="44" t="n"/>
+      <c r="I5" s="44" t="n">
+        <v>6390</v>
+      </c>
       <c r="J5" s="45" t="n"/>
       <c r="K5" s="45" t="n"/>
       <c r="L5" s="43" t="inlineStr">
@@ -8310,6 +8418,7 @@
       <c r="CP5" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ5" s="51" t="n"/>
     </row>
     <row r="6" ht="46.25" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -8352,7 +8461,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I6" s="44" t="n"/>
+      <c r="I6" s="44" t="n">
+        <v>9680</v>
+      </c>
       <c r="J6" s="45" t="n"/>
       <c r="K6" s="45" t="n"/>
       <c r="L6" s="43" t="inlineStr">
@@ -8619,6 +8730,7 @@
       <c r="CP6" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ6" s="43" t="n"/>
     </row>
     <row r="7" ht="46.25" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -8661,7 +8773,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I7" s="44" t="n"/>
+      <c r="I7" s="44" t="n">
+        <v>6490</v>
+      </c>
       <c r="J7" s="45" t="n"/>
       <c r="K7" s="45" t="n"/>
       <c r="L7" s="43" t="inlineStr">
@@ -8930,6 +9044,7 @@
       <c r="CP7" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ7" s="43" t="n"/>
     </row>
     <row r="8" ht="46.25" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -8972,7 +9087,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I8" s="44" t="n"/>
+      <c r="I8" s="44" t="n">
+        <v>10500</v>
+      </c>
       <c r="J8" s="45" t="n"/>
       <c r="K8" s="45" t="n"/>
       <c r="L8" s="43" t="inlineStr">
@@ -9241,6 +9358,7 @@
       <c r="CP8" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ8" s="43" t="n"/>
     </row>
     <row r="9" ht="46.25" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -9283,7 +9401,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I9" s="44" t="n"/>
+      <c r="I9" s="44" t="n">
+        <v>14300</v>
+      </c>
       <c r="J9" s="45" t="n"/>
       <c r="K9" s="45" t="n"/>
       <c r="L9" s="43" t="inlineStr">
@@ -9552,6 +9672,7 @@
       <c r="CP9" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ9" s="43" t="n"/>
     </row>
     <row r="10" ht="46.25" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -9594,7 +9715,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I10" s="44" t="n"/>
+      <c r="I10" s="44" t="n">
+        <v>14300</v>
+      </c>
       <c r="J10" s="45" t="n"/>
       <c r="K10" s="45" t="n"/>
       <c r="L10" s="43" t="inlineStr">
@@ -9863,6 +9986,7 @@
       <c r="CP10" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ10" s="43" t="n"/>
     </row>
     <row r="11" ht="46.25" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -9905,7 +10029,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I11" s="44" t="n"/>
+      <c r="I11" s="44" t="n">
+        <v>28700</v>
+      </c>
       <c r="J11" s="45" t="n"/>
       <c r="K11" s="45" t="n"/>
       <c r="L11" s="43" t="inlineStr">
@@ -10178,6 +10304,7 @@
       <c r="CP11" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ11" s="51" t="n"/>
     </row>
     <row r="12" ht="46.25" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -10220,7 +10347,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I12" s="44" t="n"/>
+      <c r="I12" s="44" t="n">
+        <v>20600</v>
+      </c>
       <c r="J12" s="45" t="n"/>
       <c r="K12" s="45" t="n"/>
       <c r="L12" s="43" t="inlineStr">
@@ -10489,6 +10618,7 @@
       <c r="CP12" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ12" s="43" t="n"/>
     </row>
     <row r="13" ht="46.25" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -10531,7 +10661,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I13" s="44" t="n"/>
+      <c r="I13" s="44" t="n">
+        <v>23200</v>
+      </c>
       <c r="J13" s="45" t="n"/>
       <c r="K13" s="45" t="n"/>
       <c r="L13" s="43" t="inlineStr">
@@ -10800,6 +10932,7 @@
       <c r="CP13" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ13" s="43" t="n"/>
     </row>
     <row r="14" ht="46.25" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -10842,7 +10975,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I14" s="44" t="n"/>
+      <c r="I14" s="44" t="n">
+        <v>33400</v>
+      </c>
       <c r="J14" s="45" t="n"/>
       <c r="K14" s="45" t="n"/>
       <c r="L14" s="43" t="inlineStr">
@@ -11111,6 +11246,7 @@
       <c r="CP14" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ14" s="43" t="n"/>
     </row>
     <row r="15" ht="46.25" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -11153,7 +11289,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I15" s="44" t="n"/>
+      <c r="I15" s="44" t="n">
+        <v>56300</v>
+      </c>
       <c r="J15" s="45" t="n"/>
       <c r="K15" s="45" t="n"/>
       <c r="L15" s="43" t="inlineStr">
@@ -11426,6 +11564,7 @@
       <c r="CP15" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ15" s="51" t="n"/>
     </row>
     <row r="16" ht="46.25" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -11468,7 +11607,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I16" s="44" t="n"/>
+      <c r="I16" s="44" t="n">
+        <v>10500</v>
+      </c>
       <c r="J16" s="45" t="n"/>
       <c r="K16" s="45" t="n"/>
       <c r="L16" s="43" t="inlineStr">
@@ -11728,6 +11869,7 @@
       <c r="CP16" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ16" s="43" t="n"/>
     </row>
     <row r="17" ht="46.25" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -11770,7 +11912,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I17" s="44" t="n"/>
+      <c r="I17" s="44" t="n">
+        <v>12800</v>
+      </c>
       <c r="J17" s="45" t="n"/>
       <c r="K17" s="45" t="n"/>
       <c r="L17" s="43" t="inlineStr">
@@ -12040,6 +12184,7 @@
       <c r="CP17" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ17" s="51" t="n"/>
     </row>
     <row r="18" ht="46.25" customHeight="1" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -12082,7 +12227,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I18" s="44" t="n"/>
+      <c r="I18" s="44" t="n">
+        <v>25000</v>
+      </c>
       <c r="J18" s="45" t="n"/>
       <c r="K18" s="45" t="n"/>
       <c r="L18" s="43" t="inlineStr">
@@ -12353,6 +12500,7 @@
       <c r="CP18" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ18" s="43" t="n"/>
     </row>
     <row r="19" ht="46.25" customHeight="1" s="29">
       <c r="A19" s="43" t="inlineStr">
@@ -12395,7 +12543,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I19" s="44" t="n"/>
+      <c r="I19" s="44" t="n">
+        <v>35800</v>
+      </c>
       <c r="J19" s="45" t="n"/>
       <c r="K19" s="45" t="n"/>
       <c r="L19" s="43" t="inlineStr">
@@ -12666,6 +12816,7 @@
       <c r="CP19" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ19" s="43" t="n"/>
     </row>
     <row r="20" ht="46.25" customHeight="1" s="29">
       <c r="A20" s="43" t="inlineStr">
@@ -12708,7 +12859,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I20" s="44" t="n"/>
+      <c r="I20" s="44" t="n">
+        <v>29200</v>
+      </c>
       <c r="J20" s="45" t="n"/>
       <c r="K20" s="45" t="n"/>
       <c r="L20" s="43" t="inlineStr">
@@ -12987,6 +13140,7 @@
       <c r="CP20" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ20" s="51" t="n"/>
     </row>
     <row r="21" ht="46.25" customHeight="1" s="29">
       <c r="A21" s="43" t="inlineStr">
@@ -13029,7 +13183,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I21" s="44" t="n"/>
+      <c r="I21" s="44" t="n">
+        <v>43400</v>
+      </c>
       <c r="J21" s="45" t="n"/>
       <c r="K21" s="45" t="n"/>
       <c r="L21" s="43" t="inlineStr">
@@ -13304,6 +13460,7 @@
       <c r="CP21" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ21" s="43" t="n"/>
     </row>
     <row r="22" ht="46.25" customHeight="1" s="29">
       <c r="A22" s="43" t="inlineStr">
@@ -13346,7 +13503,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I22" s="44" t="n"/>
+      <c r="I22" s="44" t="n">
+        <v>54200</v>
+      </c>
       <c r="J22" s="45" t="n"/>
       <c r="K22" s="45" t="n"/>
       <c r="L22" s="43" t="inlineStr">
@@ -13625,6 +13784,7 @@
       <c r="CP22" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ22" s="51" t="n"/>
     </row>
     <row r="23" ht="46.25" customHeight="1" s="29">
       <c r="A23" s="43" t="inlineStr">
@@ -13667,7 +13827,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I23" s="44" t="n"/>
+      <c r="I23" s="44" t="n">
+        <v>40100</v>
+      </c>
       <c r="J23" s="45" t="n"/>
       <c r="K23" s="45" t="n"/>
       <c r="L23" s="43" t="inlineStr">
@@ -13935,6 +14097,7 @@
       <c r="CP23" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ23" s="43" t="n"/>
     </row>
     <row r="24" ht="46.25" customHeight="1" s="29">
       <c r="A24" s="43" t="inlineStr">
@@ -13977,7 +14140,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I24" s="44" t="n"/>
+      <c r="I24" s="44" t="n">
+        <v>21300</v>
+      </c>
       <c r="J24" s="45" t="n"/>
       <c r="K24" s="45" t="n"/>
       <c r="L24" s="43" t="inlineStr">
@@ -14241,6 +14406,7 @@
       <c r="CP24" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ24" s="43" t="n"/>
     </row>
     <row r="25" ht="46.25" customHeight="1" s="29">
       <c r="A25" s="43" t="inlineStr">
@@ -14283,7 +14449,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I25" s="44" t="n"/>
+      <c r="I25" s="44" t="n">
+        <v>29000</v>
+      </c>
       <c r="J25" s="45" t="n"/>
       <c r="K25" s="45" t="n"/>
       <c r="L25" s="43" t="inlineStr">
@@ -14547,6 +14715,7 @@
       <c r="CP25" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ25" s="43" t="n"/>
     </row>
     <row r="26" ht="46.25" customHeight="1" s="29">
       <c r="A26" s="43" t="inlineStr">
@@ -14589,7 +14758,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I26" s="44" t="n"/>
+      <c r="I26" s="44" t="n">
+        <v>43400</v>
+      </c>
       <c r="J26" s="45" t="n"/>
       <c r="K26" s="45" t="n"/>
       <c r="L26" s="43" t="inlineStr">
@@ -14864,6 +15035,7 @@
       <c r="CP26" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ26" s="43" t="n"/>
     </row>
     <row r="27" ht="46.25" customHeight="1" s="29">
       <c r="A27" s="43" t="inlineStr">
@@ -14906,7 +15078,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I27" s="44" t="n"/>
+      <c r="I27" s="44" t="n">
+        <v>32500</v>
+      </c>
       <c r="J27" s="45" t="n"/>
       <c r="K27" s="45" t="n"/>
       <c r="L27" s="43" t="inlineStr">
@@ -15174,6 +15348,7 @@
       <c r="CP27" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ27" s="43" t="n"/>
     </row>
     <row r="28" ht="46.25" customHeight="1" s="29">
       <c r="A28" s="43" t="inlineStr">
@@ -15216,7 +15391,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I28" s="44" t="n"/>
+      <c r="I28" s="44" t="n">
+        <v>75900</v>
+      </c>
       <c r="J28" s="45" t="n"/>
       <c r="K28" s="45" t="n"/>
       <c r="L28" s="43" t="inlineStr">
@@ -15491,6 +15668,7 @@
       <c r="CP28" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ28" s="43" t="n"/>
     </row>
     <row r="29" ht="46.25" customHeight="1" s="29">
       <c r="A29" s="43" t="inlineStr">
@@ -15533,7 +15711,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I29" s="44" t="n"/>
+      <c r="I29" s="44" t="n">
+        <v>65100</v>
+      </c>
       <c r="J29" s="45" t="n"/>
       <c r="K29" s="45" t="n"/>
       <c r="L29" s="43" t="inlineStr">
@@ -15808,6 +15988,7 @@
       <c r="CP29" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ29" s="43" t="n"/>
     </row>
     <row r="30" ht="46.25" customHeight="1" s="29">
       <c r="A30" s="43" t="inlineStr">
@@ -15850,7 +16031,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I30" s="44" t="n"/>
+      <c r="I30" s="44" t="n">
+        <v>54200</v>
+      </c>
       <c r="J30" s="45" t="n"/>
       <c r="K30" s="45" t="n"/>
       <c r="L30" s="43" t="inlineStr">
@@ -16118,6 +16301,7 @@
       <c r="CP30" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ30" s="43" t="n"/>
     </row>
     <row r="31" ht="46.25" customHeight="1" s="29">
       <c r="A31" s="43" t="inlineStr">
@@ -16160,7 +16344,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I31" s="44" t="n"/>
+      <c r="I31" s="44" t="n">
+        <v>87100</v>
+      </c>
       <c r="J31" s="45" t="n"/>
       <c r="K31" s="45" t="n"/>
       <c r="L31" s="43" t="inlineStr">
@@ -16428,6 +16614,7 @@
       <c r="CP31" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ31" s="43" t="n"/>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="29">
       <c r="A32" s="43" t="inlineStr">
@@ -16470,7 +16657,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I32" s="44" t="n"/>
+      <c r="I32" s="44" t="n">
+        <v>116000</v>
+      </c>
       <c r="J32" s="45" t="n"/>
       <c r="K32" s="45" t="n"/>
       <c r="L32" s="43" t="inlineStr">
@@ -16745,6 +16934,7 @@
       <c r="CP32" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ32" s="43" t="n"/>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="29">
       <c r="A33" s="43" t="inlineStr">
@@ -16787,7 +16977,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I33" s="44" t="n"/>
+      <c r="I33" s="44" t="n">
+        <v>77400</v>
+      </c>
       <c r="J33" s="45" t="n"/>
       <c r="K33" s="45" t="n"/>
       <c r="L33" s="43" t="inlineStr">
@@ -17055,6 +17247,7 @@
       <c r="CP33" s="43" t="n">
         <v>0</v>
       </c>
+      <c r="CQ33" s="43" t="n"/>
     </row>
     <row r="34" ht="57.45" customHeight="1" s="29">
       <c r="A34" s="43" t="inlineStr">
@@ -17097,7 +17290,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I34" s="44" t="n"/>
+      <c r="I34" s="44" t="n">
+        <v>8130</v>
+      </c>
       <c r="J34" s="45" t="n"/>
       <c r="K34" s="45" t="n"/>
       <c r="L34" s="43" t="inlineStr">
@@ -17332,6 +17527,7 @@
       <c r="CP34" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ34" s="51" t="n"/>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="29">
       <c r="A35" s="43" t="inlineStr">
@@ -17374,7 +17570,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I35" s="44" t="n"/>
+      <c r="I35" s="44" t="n">
+        <v>7650</v>
+      </c>
       <c r="J35" s="45" t="n"/>
       <c r="K35" s="45" t="n"/>
       <c r="L35" s="43" t="inlineStr">
@@ -17595,6 +17793,7 @@
       <c r="CP35" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ35" s="51" t="n"/>
     </row>
     <row r="36" ht="46.25" customHeight="1" s="29">
       <c r="A36" s="43" t="inlineStr">
@@ -17637,7 +17836,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I36" s="44" t="n"/>
+      <c r="I36" s="44" t="n">
+        <v>11800</v>
+      </c>
       <c r="J36" s="45" t="n"/>
       <c r="K36" s="45" t="n"/>
       <c r="L36" s="43" t="inlineStr">
@@ -17858,6 +18059,7 @@
       <c r="CP36" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ36" s="51" t="n"/>
     </row>
     <row r="37" ht="46.25" customHeight="1" s="29">
       <c r="A37" s="43" t="inlineStr">
@@ -17900,7 +18102,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I37" s="44" t="n"/>
+      <c r="I37" s="44" t="n">
+        <v>219000</v>
+      </c>
       <c r="J37" s="45" t="n"/>
       <c r="K37" s="45" t="n"/>
       <c r="L37" s="43" t="inlineStr">
@@ -18166,6 +18370,7 @@
       <c r="CP37" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ37" s="51" t="n"/>
     </row>
     <row r="38" ht="46.25" customHeight="1" s="29">
       <c r="A38" s="43" t="inlineStr">
@@ -18208,7 +18413,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I38" s="44" t="n"/>
+      <c r="I38" s="44" t="n">
+        <v>172000</v>
+      </c>
       <c r="J38" s="45" t="n"/>
       <c r="K38" s="45" t="n"/>
       <c r="L38" s="43" t="inlineStr">
@@ -18474,6 +18681,7 @@
       <c r="CP38" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ38" s="51" t="n"/>
     </row>
     <row r="39" ht="46.25" customHeight="1" s="29">
       <c r="A39" s="43" t="inlineStr">
@@ -18516,7 +18724,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I39" s="44" t="n"/>
+      <c r="I39" s="44" t="n">
+        <v>89900</v>
+      </c>
       <c r="J39" s="45" t="n"/>
       <c r="K39" s="45" t="n"/>
       <c r="L39" s="43" t="inlineStr">
@@ -18784,6 +18994,7 @@
       <c r="CP39" s="51" t="n">
         <v>0</v>
       </c>
+      <c r="CQ39" s="51" t="n"/>
     </row>
     <row r="40" ht="46.25" customHeight="1" s="29">
       <c r="A40" s="43" t="inlineStr">
@@ -18826,7 +19037,9 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="I40" s="44" t="n"/>
+      <c r="I40" s="44" t="n">
+        <v>62900</v>
+      </c>
       <c r="J40" s="45" t="n"/>
       <c r="K40" s="45" t="n"/>
       <c r="L40" s="43" t="inlineStr">
@@ -19105,11 +19318,12 @@
       <c r="CP40" s="51" t="n">
         <v>8</v>
       </c>
+      <c r="CQ40" s="51" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:CP1"/>
-    <mergeCell ref="A2:CP2"/>
+    <mergeCell ref="A2:CQ2"/>
+    <mergeCell ref="A1:CQ1"/>
   </mergeCells>
   <dataValidations count="8">
     <dataValidation sqref="E5:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
@@ -24292,7 +24506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q131"/>
+  <dimension ref="A1:S131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="28" min="1" max="1"/>
@@ -24310,6 +24524,8 @@
     <col width="8" customWidth="1" style="28" min="14" max="15"/>
     <col width="30" customWidth="1" style="28" min="16" max="16"/>
     <col width="34" customWidth="1" style="28" min="17" max="17"/>
+    <col width="14" customWidth="1" style="29" min="18" max="18"/>
+    <col width="40" customWidth="1" style="29" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -24410,6 +24626,16 @@
       <c r="Q4" s="42" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="R4" s="42" t="inlineStr">
+        <is>
+          <t>Cost_Index</t>
+        </is>
+      </c>
+      <c r="S4" s="42" t="inlineStr">
+        <is>
+          <t>Cost_Note</t>
         </is>
       </c>
     </row>
@@ -24475,6 +24701,10 @@
         </is>
       </c>
       <c r="Q5" s="43" t="n"/>
+      <c r="R5" s="43" t="n">
+        <v>1370</v>
+      </c>
+      <c r="S5" s="43" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -24538,6 +24768,10 @@
         </is>
       </c>
       <c r="Q6" s="43" t="n"/>
+      <c r="R6" s="43" t="n">
+        <v>2880</v>
+      </c>
+      <c r="S6" s="43" t="n"/>
     </row>
     <row r="7" ht="23.85" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -24605,6 +24839,10 @@
           <t>M4250-16XF: ports 1-12 only</t>
         </is>
       </c>
+      <c r="R7" s="43" t="n">
+        <v>1370</v>
+      </c>
+      <c r="S7" s="43" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -24668,6 +24906,10 @@
         </is>
       </c>
       <c r="Q8" s="43" t="n"/>
+      <c r="R8" s="43" t="n">
+        <v>3600</v>
+      </c>
+      <c r="S8" s="43" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -24735,6 +24977,8 @@
           <t>Qty 10 per SKU</t>
         </is>
       </c>
+      <c r="R9" s="43" t="n"/>
+      <c r="S9" s="43" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -24798,6 +25042,10 @@
         </is>
       </c>
       <c r="Q10" s="43" t="n"/>
+      <c r="R10" s="43" t="n">
+        <v>8630</v>
+      </c>
+      <c r="S10" s="43" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -24865,6 +25113,8 @@
           <t>Qty 10 per SKU</t>
         </is>
       </c>
+      <c r="R11" s="43" t="n"/>
+      <c r="S11" s="43" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -24928,6 +25178,10 @@
         </is>
       </c>
       <c r="Q12" s="43" t="n"/>
+      <c r="R12" s="43" t="n">
+        <v>3600</v>
+      </c>
+      <c r="S12" s="43" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -24991,6 +25245,10 @@
         </is>
       </c>
       <c r="Q13" s="43" t="n"/>
+      <c r="R13" s="43" t="n">
+        <v>3600</v>
+      </c>
+      <c r="S13" s="43" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -25054,6 +25312,10 @@
         </is>
       </c>
       <c r="Q14" s="43" t="n"/>
+      <c r="R14" s="43" t="n">
+        <v>3430</v>
+      </c>
+      <c r="S14" s="43" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -25113,6 +25375,10 @@
         </is>
       </c>
       <c r="Q15" s="43" t="n"/>
+      <c r="R15" s="43" t="n">
+        <v>535</v>
+      </c>
+      <c r="S15" s="43" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -25172,6 +25438,10 @@
         </is>
       </c>
       <c r="Q16" s="43" t="n"/>
+      <c r="R16" s="43" t="n">
+        <v>802</v>
+      </c>
+      <c r="S16" s="43" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -25231,6 +25501,10 @@
         </is>
       </c>
       <c r="Q17" s="43" t="n"/>
+      <c r="R17" s="43" t="n">
+        <v>1070</v>
+      </c>
+      <c r="S17" s="43" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -25290,6 +25564,10 @@
         </is>
       </c>
       <c r="Q18" s="43" t="n"/>
+      <c r="R18" s="43" t="n">
+        <v>396</v>
+      </c>
+      <c r="S18" s="43" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="29">
       <c r="A19" s="43" t="inlineStr">
@@ -25349,6 +25627,10 @@
         </is>
       </c>
       <c r="Q19" s="43" t="n"/>
+      <c r="R19" s="43" t="n">
+        <v>428</v>
+      </c>
+      <c r="S19" s="43" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="29">
       <c r="A20" s="43" t="inlineStr">
@@ -25408,6 +25690,10 @@
         </is>
       </c>
       <c r="Q20" s="43" t="n"/>
+      <c r="R20" s="43" t="n">
+        <v>503</v>
+      </c>
+      <c r="S20" s="43" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="29">
       <c r="A21" s="43" t="inlineStr">
@@ -25467,6 +25753,10 @@
         </is>
       </c>
       <c r="Q21" s="43" t="n"/>
+      <c r="R21" s="43" t="n">
+        <v>588</v>
+      </c>
+      <c r="S21" s="43" t="n"/>
     </row>
     <row r="22" ht="46.25" customHeight="1" s="29">
       <c r="A22" s="43" t="inlineStr">
@@ -25526,6 +25816,10 @@
           <t>For M4350-8M2V and M4250-8G2XF-PoE+</t>
         </is>
       </c>
+      <c r="R22" s="43" t="n">
+        <v>2900</v>
+      </c>
+      <c r="S22" s="43" t="n"/>
     </row>
     <row r="23" ht="46.25" customHeight="1" s="29">
       <c r="A23" s="43" t="inlineStr">
@@ -25585,6 +25879,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R23" s="43" t="n">
+        <v>2900</v>
+      </c>
+      <c r="S23" s="43" t="n"/>
     </row>
     <row r="24" ht="46.25" customHeight="1" s="29">
       <c r="A24" s="43" t="inlineStr">
@@ -25644,6 +25942,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R24" s="43" t="n">
+        <v>2900</v>
+      </c>
+      <c r="S24" s="43" t="n"/>
     </row>
     <row r="25" ht="46.25" customHeight="1" s="29">
       <c r="A25" s="43" t="inlineStr">
@@ -25703,6 +26005,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R25" s="43" t="n">
+        <v>2900</v>
+      </c>
+      <c r="S25" s="43" t="n"/>
     </row>
     <row r="26" ht="46.25" customHeight="1" s="29">
       <c r="A26" s="43" t="inlineStr">
@@ -25762,6 +26068,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R26" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S26" s="43" t="n"/>
     </row>
     <row r="27" ht="46.25" customHeight="1" s="29">
       <c r="A27" s="43" t="inlineStr">
@@ -25821,6 +26131,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R27" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S27" s="43" t="n"/>
     </row>
     <row r="28" ht="46.25" customHeight="1" s="29">
       <c r="A28" s="43" t="inlineStr">
@@ -25880,6 +26194,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R28" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S28" s="43" t="n"/>
     </row>
     <row r="29" ht="46.25" customHeight="1" s="29">
       <c r="A29" s="43" t="inlineStr">
@@ -25939,6 +26257,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R29" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S29" s="43" t="n"/>
     </row>
     <row r="30" ht="46.25" customHeight="1" s="29">
       <c r="A30" s="43" t="inlineStr">
@@ -25998,6 +26320,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R30" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S30" s="43" t="n"/>
     </row>
     <row r="31" ht="46.25" customHeight="1" s="29">
       <c r="A31" s="43" t="inlineStr">
@@ -26057,6 +26383,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R31" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S31" s="43" t="n"/>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="29">
       <c r="A32" s="43" t="inlineStr">
@@ -26116,6 +26446,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R32" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S32" s="43" t="n"/>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="29">
       <c r="A33" s="43" t="inlineStr">
@@ -26175,6 +26509,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R33" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S33" s="43" t="n"/>
     </row>
     <row r="34" ht="46.25" customHeight="1" s="29">
       <c r="A34" s="43" t="inlineStr">
@@ -26234,6 +26572,10 @@
           <t>PSU group A</t>
         </is>
       </c>
+      <c r="R34" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S34" s="43" t="n"/>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="29">
       <c r="A35" s="43" t="inlineStr">
@@ -26293,6 +26635,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R35" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S35" s="43" t="n"/>
     </row>
     <row r="36" ht="46.25" customHeight="1" s="29">
       <c r="A36" s="43" t="inlineStr">
@@ -26352,6 +26698,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R36" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S36" s="43" t="n"/>
     </row>
     <row r="37" ht="46.25" customHeight="1" s="29">
       <c r="A37" s="43" t="inlineStr">
@@ -26411,6 +26761,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R37" s="43" t="n">
+        <v>3390</v>
+      </c>
+      <c r="S37" s="43" t="n"/>
     </row>
     <row r="38" ht="46.25" customHeight="1" s="29">
       <c r="A38" s="43" t="inlineStr">
@@ -26470,6 +26824,10 @@
           <t>PSU group B; PoE matrix shows lower budget at 110VAC - datasheet does not state 110V rating</t>
         </is>
       </c>
+      <c r="R38" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S38" s="43" t="n"/>
     </row>
     <row r="39" ht="46.25" customHeight="1" s="29">
       <c r="A39" s="43" t="inlineStr">
@@ -26529,6 +26887,10 @@
           <t>PSU group B; PoE matrix shows lower budget at 110VAC - datasheet does not state 110V rating</t>
         </is>
       </c>
+      <c r="R39" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S39" s="43" t="n"/>
     </row>
     <row r="40" ht="46.25" customHeight="1" s="29">
       <c r="A40" s="43" t="inlineStr">
@@ -26588,6 +26950,10 @@
           <t>PSU group B; PoE matrix shows lower budget at 110VAC - datasheet does not state 110V rating</t>
         </is>
       </c>
+      <c r="R40" s="43" t="n">
+        <v>4360</v>
+      </c>
+      <c r="S40" s="43" t="n"/>
     </row>
     <row r="41" ht="46.25" customHeight="1" s="29">
       <c r="A41" s="43" t="inlineStr">
@@ -26647,6 +27013,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R41" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S41" s="43" t="n"/>
     </row>
     <row r="42" ht="46.25" customHeight="1" s="29">
       <c r="A42" s="43" t="inlineStr">
@@ -26706,6 +27076,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R42" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S42" s="43" t="n"/>
     </row>
     <row r="43" ht="46.25" customHeight="1" s="29">
       <c r="A43" s="43" t="inlineStr">
@@ -26765,6 +27139,10 @@
           <t>PSU group B</t>
         </is>
       </c>
+      <c r="R43" s="43" t="n">
+        <v>7260</v>
+      </c>
+      <c r="S43" s="43" t="n"/>
     </row>
     <row r="44" ht="46.25" customHeight="1" s="29">
       <c r="A44" s="43" t="inlineStr">
@@ -26804,6 +27182,10 @@
         </is>
       </c>
       <c r="Q44" s="43" t="n"/>
+      <c r="R44" s="43" t="n">
+        <v>2900</v>
+      </c>
+      <c r="S44" s="43" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="29">
       <c r="A45" s="43" t="inlineStr">
@@ -26849,6 +27231,8 @@
           <t>SKUs marked WIP in datasheet</t>
         </is>
       </c>
+      <c r="R45" s="43" t="n"/>
+      <c r="S45" s="43" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="29">
       <c r="A46" s="43" t="inlineStr">
@@ -26894,6 +27278,8 @@
           <t>SKUs marked WIP in datasheet</t>
         </is>
       </c>
+      <c r="R46" s="43" t="n"/>
+      <c r="S46" s="43" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="29">
       <c r="A47" s="43" t="inlineStr">
@@ -26939,6 +27325,8 @@
           <t>SKUs marked WIP in datasheet</t>
         </is>
       </c>
+      <c r="R47" s="43" t="n"/>
+      <c r="S47" s="43" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="29">
       <c r="A48" s="43" t="inlineStr">
@@ -26984,6 +27372,8 @@
           <t>SKUs marked WIP in datasheet</t>
         </is>
       </c>
+      <c r="R48" s="43" t="n"/>
+      <c r="S48" s="43" t="n"/>
     </row>
     <row r="49" ht="23.85" customHeight="1" s="29">
       <c r="A49" s="43" t="inlineStr">
@@ -27027,6 +27417,8 @@
           <t>All M4250 models</t>
         </is>
       </c>
+      <c r="R49" s="43" t="n"/>
+      <c r="S49" s="43" t="n"/>
     </row>
     <row r="50" ht="23.85" customHeight="1" s="29">
       <c r="A50" s="43" t="inlineStr">
@@ -27072,6 +27464,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R50" s="43" t="n"/>
+      <c r="S50" s="43" t="n"/>
     </row>
     <row r="51" ht="23.85" customHeight="1" s="29">
       <c r="A51" s="43" t="inlineStr">
@@ -27117,6 +27511,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R51" s="43" t="n"/>
+      <c r="S51" s="43" t="n"/>
     </row>
     <row r="52" ht="23.85" customHeight="1" s="29">
       <c r="A52" s="43" t="inlineStr">
@@ -27162,6 +27558,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R52" s="43" t="n"/>
+      <c r="S52" s="43" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="29">
       <c r="A53" s="43" t="inlineStr">
@@ -27207,6 +27605,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R53" s="43" t="n"/>
+      <c r="S53" s="43" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="29">
       <c r="A54" s="43" t="inlineStr">
@@ -27252,6 +27652,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R54" s="43" t="n"/>
+      <c r="S54" s="43" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="29">
       <c r="A55" s="43" t="inlineStr">
@@ -27297,6 +27699,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R55" s="43" t="n"/>
+      <c r="S55" s="43" t="n"/>
     </row>
     <row r="56" ht="46.25" customHeight="1" s="29">
       <c r="A56" s="43" t="inlineStr">
@@ -27342,6 +27746,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R56" s="43" t="n"/>
+      <c r="S56" s="43" t="n"/>
     </row>
     <row r="57" ht="46.25" customHeight="1" s="29">
       <c r="A57" s="43" t="inlineStr">
@@ -27387,6 +27793,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R57" s="43" t="n"/>
+      <c r="S57" s="43" t="n"/>
     </row>
     <row r="58" ht="46.25" customHeight="1" s="29">
       <c r="A58" s="43" t="inlineStr">
@@ -27432,6 +27840,8 @@
           <t>Legacy OnCall (ProSupport): not sold for products purchased after 2026-04-13; replaced by Sprint / Overdrive / Fastlane. Not used by the tool</t>
         </is>
       </c>
+      <c r="R58" s="43" t="n"/>
+      <c r="S58" s="43" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="29">
       <c r="A59" s="43" t="inlineStr">
@@ -27473,6 +27883,8 @@
         </is>
       </c>
       <c r="Q59" s="43" t="n"/>
+      <c r="R59" s="43" t="n"/>
+      <c r="S59" s="43" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="29">
       <c r="A60" s="43" t="inlineStr">
@@ -27514,6 +27926,8 @@
         </is>
       </c>
       <c r="Q60" s="43" t="n"/>
+      <c r="R60" s="43" t="n"/>
+      <c r="S60" s="43" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="29">
       <c r="A61" s="43" t="inlineStr">
@@ -27555,6 +27969,8 @@
         </is>
       </c>
       <c r="Q61" s="43" t="n"/>
+      <c r="R61" s="43" t="n"/>
+      <c r="S61" s="43" t="n"/>
     </row>
     <row r="62" ht="23.85" customHeight="1" s="29">
       <c r="A62" s="43" t="inlineStr">
@@ -27596,6 +28012,8 @@
         </is>
       </c>
       <c r="Q62" s="43" t="n"/>
+      <c r="R62" s="43" t="n"/>
+      <c r="S62" s="43" t="n"/>
     </row>
     <row r="63" ht="23.85" customHeight="1" s="29">
       <c r="A63" s="43" t="inlineStr">
@@ -27637,6 +28055,8 @@
         </is>
       </c>
       <c r="Q63" s="43" t="n"/>
+      <c r="R63" s="43" t="n"/>
+      <c r="S63" s="43" t="n"/>
     </row>
     <row r="64" ht="23.85" customHeight="1" s="29">
       <c r="A64" s="43" t="inlineStr">
@@ -27678,6 +28098,8 @@
         </is>
       </c>
       <c r="Q64" s="43" t="n"/>
+      <c r="R64" s="43" t="n"/>
+      <c r="S64" s="43" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="29">
       <c r="A65" s="43" t="inlineStr">
@@ -27719,6 +28141,8 @@
         </is>
       </c>
       <c r="Q65" s="43" t="n"/>
+      <c r="R65" s="43" t="n"/>
+      <c r="S65" s="43" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="29">
       <c r="A66" s="43" t="inlineStr">
@@ -27760,6 +28184,8 @@
         </is>
       </c>
       <c r="Q66" s="43" t="n"/>
+      <c r="R66" s="43" t="n"/>
+      <c r="S66" s="43" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="29">
       <c r="A67" s="43" t="inlineStr">
@@ -27801,6 +28227,8 @@
         </is>
       </c>
       <c r="Q67" s="43" t="n"/>
+      <c r="R67" s="43" t="n"/>
+      <c r="S67" s="43" t="n"/>
     </row>
     <row r="68" ht="23.85" customHeight="1" s="29">
       <c r="A68" s="43" t="inlineStr">
@@ -27842,6 +28270,8 @@
         </is>
       </c>
       <c r="Q68" s="43" t="n"/>
+      <c r="R68" s="43" t="n"/>
+      <c r="S68" s="43" t="n"/>
     </row>
     <row r="69" ht="23.85" customHeight="1" s="29">
       <c r="A69" s="43" t="inlineStr">
@@ -27883,6 +28313,8 @@
         </is>
       </c>
       <c r="Q69" s="43" t="n"/>
+      <c r="R69" s="43" t="n"/>
+      <c r="S69" s="43" t="n"/>
     </row>
     <row r="70" ht="23.85" customHeight="1" s="29">
       <c r="A70" s="43" t="inlineStr">
@@ -27924,6 +28356,8 @@
         </is>
       </c>
       <c r="Q70" s="43" t="n"/>
+      <c r="R70" s="43" t="n"/>
+      <c r="S70" s="43" t="n"/>
     </row>
     <row r="71" ht="23.85" customHeight="1" s="29">
       <c r="A71" s="43" t="inlineStr">
@@ -27991,6 +28425,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca</t>
         </is>
       </c>
+      <c r="R71" s="43" t="n">
+        <v>3510</v>
+      </c>
+      <c r="S71" s="43" t="n"/>
     </row>
     <row r="72" ht="23.85" customHeight="1" s="29">
       <c r="A72" s="43" t="inlineStr">
@@ -28058,6 +28496,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca</t>
         </is>
       </c>
+      <c r="R72" s="43" t="n">
+        <v>8050</v>
+      </c>
+      <c r="S72" s="43" t="n"/>
     </row>
     <row r="73" ht="23.85" customHeight="1" s="29">
       <c r="A73" s="43" t="inlineStr">
@@ -28125,6 +28567,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca</t>
         </is>
       </c>
+      <c r="R73" s="43" t="n">
+        <v>7300</v>
+      </c>
+      <c r="S73" s="43" t="n"/>
     </row>
     <row r="74" ht="23.85" customHeight="1" s="29">
       <c r="A74" s="43" t="inlineStr">
@@ -28192,6 +28638,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca</t>
         </is>
       </c>
+      <c r="R74" s="43" t="n">
+        <v>6820</v>
+      </c>
+      <c r="S74" s="43" t="n"/>
     </row>
     <row r="75" ht="23.85" customHeight="1" s="29">
       <c r="A75" s="43" t="inlineStr">
@@ -28259,6 +28709,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca</t>
         </is>
       </c>
+      <c r="R75" s="43" t="n">
+        <v>6820</v>
+      </c>
+      <c r="S75" s="43" t="n"/>
     </row>
     <row r="76" ht="23.85" customHeight="1" s="29">
       <c r="A76" s="43" t="inlineStr">
@@ -28322,6 +28776,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R76" s="43" t="n">
+        <v>458</v>
+      </c>
+      <c r="S76" s="43" t="n"/>
     </row>
     <row r="77" ht="23.85" customHeight="1" s="29">
       <c r="A77" s="43" t="inlineStr">
@@ -28385,6 +28843,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R77" s="43" t="n">
+        <v>458</v>
+      </c>
+      <c r="S77" s="43" t="n"/>
     </row>
     <row r="78" ht="23.85" customHeight="1" s="29">
       <c r="A78" s="43" t="inlineStr">
@@ -28448,6 +28910,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R78" s="43" t="n">
+        <v>458</v>
+      </c>
+      <c r="S78" s="43" t="n"/>
     </row>
     <row r="79" ht="23.85" customHeight="1" s="29">
       <c r="A79" s="43" t="inlineStr">
@@ -28511,6 +28977,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R79" s="43" t="n">
+        <v>695</v>
+      </c>
+      <c r="S79" s="43" t="n"/>
     </row>
     <row r="80" ht="23.85" customHeight="1" s="29">
       <c r="A80" s="43" t="inlineStr">
@@ -28574,6 +29044,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R80" s="43" t="n">
+        <v>1480</v>
+      </c>
+      <c r="S80" s="43" t="n"/>
     </row>
     <row r="81" ht="23.85" customHeight="1" s="29">
       <c r="A81" s="43" t="inlineStr">
@@ -28637,6 +29111,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R81" s="43" t="n">
+        <v>1480</v>
+      </c>
+      <c r="S81" s="43" t="n"/>
     </row>
     <row r="82" ht="23.85" customHeight="1" s="29">
       <c r="A82" s="43" t="inlineStr">
@@ -28700,6 +29178,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R82" s="43" t="n">
+        <v>1480</v>
+      </c>
+      <c r="S82" s="43" t="n"/>
     </row>
     <row r="83" ht="23.85" customHeight="1" s="29">
       <c r="A83" s="43" t="inlineStr">
@@ -28763,6 +29245,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R83" s="43" t="n">
+        <v>1830</v>
+      </c>
+      <c r="S83" s="43" t="n"/>
     </row>
     <row r="84" ht="23.85" customHeight="1" s="29">
       <c r="A84" s="43" t="inlineStr">
@@ -28826,6 +29312,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R84" s="43" t="n">
+        <v>1830</v>
+      </c>
+      <c r="S84" s="43" t="n"/>
     </row>
     <row r="85" ht="23.85" customHeight="1" s="29">
       <c r="A85" s="43" t="inlineStr">
@@ -28889,6 +29379,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R85" s="43" t="n">
+        <v>1830</v>
+      </c>
+      <c r="S85" s="43" t="n"/>
     </row>
     <row r="86" ht="23.85" customHeight="1" s="29">
       <c r="A86" s="43" t="inlineStr">
@@ -28952,6 +29446,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R86" s="43" t="n">
+        <v>1190</v>
+      </c>
+      <c r="S86" s="43" t="n"/>
     </row>
     <row r="87" ht="23.85" customHeight="1" s="29">
       <c r="A87" s="43" t="inlineStr">
@@ -29015,6 +29513,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R87" s="43" t="n">
+        <v>1190</v>
+      </c>
+      <c r="S87" s="43" t="n"/>
     </row>
     <row r="88" ht="23.85" customHeight="1" s="29">
       <c r="A88" s="43" t="inlineStr">
@@ -29078,6 +29580,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R88" s="43" t="n">
+        <v>1190</v>
+      </c>
+      <c r="S88" s="43" t="n"/>
     </row>
     <row r="89" ht="23.85" customHeight="1" s="29">
       <c r="A89" s="43" t="inlineStr">
@@ -29141,6 +29647,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request</t>
         </is>
       </c>
+      <c r="R89" s="43" t="n">
+        <v>1620</v>
+      </c>
+      <c r="S89" s="43" t="n"/>
     </row>
     <row r="90" ht="23.85" customHeight="1" s="29">
       <c r="A90" s="43" t="inlineStr">
@@ -29204,6 +29714,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R90" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S90" s="43" t="n"/>
     </row>
     <row r="91" ht="23.85" customHeight="1" s="29">
       <c r="A91" s="43" t="inlineStr">
@@ -29267,6 +29781,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R91" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S91" s="43" t="n"/>
     </row>
     <row r="92" ht="23.85" customHeight="1" s="29">
       <c r="A92" s="43" t="inlineStr">
@@ -29330,6 +29848,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R92" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S92" s="43" t="n"/>
     </row>
     <row r="93" ht="23.85" customHeight="1" s="29">
       <c r="A93" s="43" t="inlineStr">
@@ -29393,6 +29915,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R93" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S93" s="43" t="n"/>
     </row>
     <row r="94" ht="23.85" customHeight="1" s="29">
       <c r="A94" s="43" t="inlineStr">
@@ -29456,6 +29982,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R94" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S94" s="43" t="n"/>
     </row>
     <row r="95" ht="23.85" customHeight="1" s="29">
       <c r="A95" s="43" t="inlineStr">
@@ -29519,6 +30049,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request</t>
         </is>
       </c>
+      <c r="R95" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S95" s="43" t="n"/>
     </row>
     <row r="96" ht="23.85" customHeight="1" s="29">
       <c r="A96" s="43" t="inlineStr">
@@ -29582,6 +30116,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R96" s="43" t="n">
+        <v>1670</v>
+      </c>
+      <c r="S96" s="43" t="n"/>
     </row>
     <row r="97" ht="23.85" customHeight="1" s="29">
       <c r="A97" s="43" t="inlineStr">
@@ -29645,6 +30183,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R97" s="43" t="n">
+        <v>1670</v>
+      </c>
+      <c r="S97" s="43" t="n"/>
     </row>
     <row r="98" ht="23.85" customHeight="1" s="29">
       <c r="A98" s="43" t="inlineStr">
@@ -29708,6 +30250,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R98" s="43" t="n">
+        <v>1670</v>
+      </c>
+      <c r="S98" s="43" t="n"/>
     </row>
     <row r="99" ht="23.85" customHeight="1" s="29">
       <c r="A99" s="43" t="inlineStr">
@@ -29771,6 +30317,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 5m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R99" s="43" t="n">
+        <v>2470</v>
+      </c>
+      <c r="S99" s="43" t="n"/>
     </row>
     <row r="100" ht="23.85" customHeight="1" s="29">
       <c r="A100" s="43" t="inlineStr">
@@ -29834,6 +30384,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R100" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S100" s="43" t="n"/>
     </row>
     <row r="101" ht="23.85" customHeight="1" s="29">
       <c r="A101" s="43" t="inlineStr">
@@ -29897,6 +30451,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R101" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S101" s="43" t="n"/>
     </row>
     <row r="102" ht="23.85" customHeight="1" s="29">
       <c r="A102" s="43" t="inlineStr">
@@ -29960,6 +30518,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R102" s="43" t="n">
+        <v>7030</v>
+      </c>
+      <c r="S102" s="43" t="n"/>
     </row>
     <row r="103" ht="23.85" customHeight="1" s="29">
       <c r="A103" s="43" t="inlineStr">
@@ -30023,6 +30585,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R103" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S103" s="43" t="n"/>
     </row>
     <row r="104" ht="23.85" customHeight="1" s="29">
       <c r="A104" s="43" t="inlineStr">
@@ -30086,6 +30652,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R104" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S104" s="43" t="n"/>
     </row>
     <row r="105" ht="23.85" customHeight="1" s="29">
       <c r="A105" s="43" t="inlineStr">
@@ -30149,6 +30719,10 @@
           <t>Third-party: optic.ca, NETGEAR certified. Order from optic.ca. Custom lengths to 30m on request. Breakout not used by engine yet</t>
         </is>
       </c>
+      <c r="R105" s="43" t="n">
+        <v>7740</v>
+      </c>
+      <c r="S105" s="43" t="n"/>
     </row>
     <row r="106" ht="23.85" customHeight="1" s="29">
       <c r="A106" s="43" t="inlineStr">
@@ -30216,6 +30790,8 @@
           <t>M4500 only (not in M4350 datasheet)</t>
         </is>
       </c>
+      <c r="R106" s="43" t="n"/>
+      <c r="S106" s="43" t="n"/>
     </row>
     <row r="107" ht="23.85" customHeight="1" s="29">
       <c r="A107" s="43" t="inlineStr">
@@ -30283,6 +30859,8 @@
           <t>M4500 only (not in M4350 datasheet)</t>
         </is>
       </c>
+      <c r="R107" s="43" t="n"/>
+      <c r="S107" s="43" t="n"/>
     </row>
     <row r="108" ht="23.85" customHeight="1" s="29">
       <c r="A108" s="43" t="inlineStr">
@@ -30346,6 +30924,8 @@
         </is>
       </c>
       <c r="Q108" s="43" t="n"/>
+      <c r="R108" s="43" t="n"/>
+      <c r="S108" s="43" t="n"/>
     </row>
     <row r="109" ht="23.85" customHeight="1" s="29">
       <c r="A109" s="43" t="inlineStr">
@@ -30409,6 +30989,8 @@
         </is>
       </c>
       <c r="Q109" s="43" t="n"/>
+      <c r="R109" s="43" t="n"/>
+      <c r="S109" s="43" t="n"/>
     </row>
     <row r="110" ht="23.85" customHeight="1" s="29">
       <c r="A110" s="43" t="inlineStr">
@@ -30468,6 +31050,8 @@
         </is>
       </c>
       <c r="Q110" s="43" t="n"/>
+      <c r="R110" s="43" t="n"/>
+      <c r="S110" s="43" t="n"/>
     </row>
     <row r="111" ht="23.85" customHeight="1" s="29">
       <c r="A111" s="43" t="inlineStr">
@@ -30527,6 +31111,8 @@
         </is>
       </c>
       <c r="Q111" s="43" t="n"/>
+      <c r="R111" s="43" t="n"/>
+      <c r="S111" s="43" t="n"/>
     </row>
     <row r="112" ht="23.85" customHeight="1" s="29">
       <c r="A112" s="43" t="inlineStr">
@@ -30586,6 +31172,8 @@
         </is>
       </c>
       <c r="Q112" s="43" t="n"/>
+      <c r="R112" s="43" t="n"/>
+      <c r="S112" s="43" t="n"/>
     </row>
     <row r="113" ht="23.85" customHeight="1" s="29">
       <c r="A113" s="43" t="inlineStr">
@@ -30645,6 +31233,8 @@
         </is>
       </c>
       <c r="Q113" s="43" t="n"/>
+      <c r="R113" s="43" t="n"/>
+      <c r="S113" s="43" t="n"/>
     </row>
     <row r="114" ht="23.85" customHeight="1" s="29">
       <c r="A114" s="43" t="inlineStr">
@@ -30700,6 +31290,8 @@
           <t>PSU group C. Spare only</t>
         </is>
       </c>
+      <c r="R114" s="43" t="n"/>
+      <c r="S114" s="43" t="n"/>
     </row>
     <row r="115" ht="23.85" customHeight="1" s="29">
       <c r="A115" s="43" t="inlineStr">
@@ -30747,6 +31339,8 @@
           <t>Spare only</t>
         </is>
       </c>
+      <c r="R115" s="43" t="n"/>
+      <c r="S115" s="43" t="n"/>
     </row>
     <row r="116" ht="23.85" customHeight="1" s="29">
       <c r="A116" s="43" t="inlineStr">
@@ -30792,6 +31386,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R116" s="43" t="n"/>
+      <c r="S116" s="43" t="n"/>
     </row>
     <row r="117" ht="23.85" customHeight="1" s="29">
       <c r="A117" s="43" t="inlineStr">
@@ -30837,6 +31433,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R117" s="43" t="n"/>
+      <c r="S117" s="43" t="n"/>
     </row>
     <row r="118" ht="23.85" customHeight="1" s="29">
       <c r="A118" s="43" t="inlineStr">
@@ -30882,6 +31480,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R118" s="43" t="n"/>
+      <c r="S118" s="43" t="n"/>
     </row>
     <row r="119" ht="23.85" customHeight="1" s="29">
       <c r="A119" s="43" t="inlineStr">
@@ -30923,6 +31523,8 @@
         </is>
       </c>
       <c r="Q119" s="43" t="n"/>
+      <c r="R119" s="43" t="n"/>
+      <c r="S119" s="43" t="n"/>
     </row>
     <row r="120" ht="23.85" customHeight="1" s="29">
       <c r="A120" s="43" t="inlineStr">
@@ -30964,6 +31566,8 @@
         </is>
       </c>
       <c r="Q120" s="43" t="n"/>
+      <c r="R120" s="43" t="n"/>
+      <c r="S120" s="43" t="n"/>
     </row>
     <row r="121" ht="23.85" customHeight="1" s="29">
       <c r="A121" s="43" t="inlineStr">
@@ -31005,6 +31609,8 @@
         </is>
       </c>
       <c r="Q121" s="43" t="n"/>
+      <c r="R121" s="43" t="n"/>
+      <c r="S121" s="43" t="n"/>
     </row>
     <row r="122" ht="23.85" customHeight="1" s="29">
       <c r="A122" s="43" t="inlineStr">
@@ -31050,6 +31656,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R122" s="43" t="n"/>
+      <c r="S122" s="43" t="n"/>
     </row>
     <row r="123" ht="23.85" customHeight="1" s="29">
       <c r="A123" s="43" t="inlineStr">
@@ -31095,6 +31703,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R123" s="43" t="n"/>
+      <c r="S123" s="43" t="n"/>
     </row>
     <row r="124" ht="23.85" customHeight="1" s="29">
       <c r="A124" s="43" t="inlineStr">
@@ -31140,6 +31750,8 @@
           <t>3-yr Sprint is included with the switch</t>
         </is>
       </c>
+      <c r="R124" s="43" t="n"/>
+      <c r="S124" s="43" t="n"/>
     </row>
     <row r="125" ht="23.85" customHeight="1" s="29">
       <c r="A125" s="43" t="inlineStr">
@@ -31181,6 +31793,8 @@
         </is>
       </c>
       <c r="Q125" s="43" t="n"/>
+      <c r="R125" s="43" t="n"/>
+      <c r="S125" s="43" t="n"/>
     </row>
     <row r="126" ht="23.85" customHeight="1" s="29">
       <c r="A126" s="43" t="inlineStr">
@@ -31222,6 +31836,8 @@
         </is>
       </c>
       <c r="Q126" s="43" t="n"/>
+      <c r="R126" s="43" t="n"/>
+      <c r="S126" s="43" t="n"/>
     </row>
     <row r="127" ht="23.85" customHeight="1" s="29">
       <c r="A127" s="43" t="inlineStr">
@@ -31263,6 +31879,8 @@
         </is>
       </c>
       <c r="Q127" s="43" t="n"/>
+      <c r="R127" s="43" t="n"/>
+      <c r="S127" s="43" t="n"/>
     </row>
     <row r="128" ht="23.85" customHeight="1" s="29">
       <c r="A128" s="43" t="inlineStr">
@@ -31318,6 +31936,10 @@
           <t>Included with MSM4320. AOC recommended for 25G (passive DAC can take 15-70 s to link)</t>
         </is>
       </c>
+      <c r="R128" s="43" t="n">
+        <v>6420</v>
+      </c>
+      <c r="S128" s="43" t="n"/>
     </row>
     <row r="129" ht="23.85" customHeight="1" s="29">
       <c r="A129" s="43" t="inlineStr">
@@ -31373,6 +31995,10 @@
           <t>Optional for MSM4320. No 100M/2.5G/5G</t>
         </is>
       </c>
+      <c r="R129" s="43" t="n">
+        <v>6420</v>
+      </c>
+      <c r="S129" s="43" t="n"/>
     </row>
     <row r="130" ht="23.85" customHeight="1" s="29">
       <c r="A130" s="43" t="inlineStr">
@@ -31432,6 +32058,10 @@
           <t>Optional for MSM4320. Includes 4 MMF patch cords to the opticalCON connectors; transceivers ordered separately</t>
         </is>
       </c>
+      <c r="R130" s="43" t="n">
+        <v>13900</v>
+      </c>
+      <c r="S130" s="43" t="n"/>
     </row>
     <row r="131" ht="23.85" customHeight="1" s="29">
       <c r="A131" s="43" t="inlineStr">
@@ -31491,11 +32121,15 @@
           <t>Optional for MSM4320. Includes 4 SMF patch cords to the opticalCON connectors; transceivers ordered separately</t>
         </is>
       </c>
+      <c r="R131" s="43" t="n">
+        <v>13900</v>
+      </c>
+      <c r="S131" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C5:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">

</xml_diff>

<commit_message>
Best design first, third-party modules for long runs, and brands in the BoM
- Design priority: Best design (default) ranks valid designs by fewest
  switches and uplinks, with a 30% cost safety net; Lowest cost is an
  internal team-mode option
- When no catalog optic reaches a distance but a third-party module type
  does (25G/100G eSR, ER/ZR), the BoM adds it as 3P-... (buy separately)
  with a warning instead of adding switches; catalog speeds still first
- Accessories get a Brand column (NETGEAR, optic.ca, future suppliers);
  brand shown in the BoM table, CSV, Excel and PDF
- Tool_Settings: Allow_Third_Party_Optics, Best_Design_Cost_Margin_Pct
- Flowcharts, docs, validation summary and reports updated
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1161,7 +1161,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F113"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Sheet"/>
@@ -1201,9 +1201,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:S131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblAccessories" displayName="tblAccessories" ref="A4:T131" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:Q127"/>
-  <tableColumns count="19">
+  <tableColumns count="20">
     <tableColumn id="1" name="Orderable_SKU"/>
     <tableColumn id="2" name="Base_Model"/>
     <tableColumn id="3" name="Category"/>
@@ -1223,6 +1223,7 @@
     <tableColumn id="17" name="Notes"/>
     <tableColumn id="18" name="Cost_Index"/>
     <tableColumn id="19" name="Cost_Note"/>
+    <tableColumn id="20" name="Brand"/>
   </tableColumns>
 </table>
 </file>
@@ -1314,7 +1315,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="tblSettings" displayName="tblSettings" ref="A4:C23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:C17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Key"/>
@@ -2699,7 +2700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="28" min="1" max="1"/>
@@ -2860,25 +2861,29 @@
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>Default_Spare_Pct</t>
+          <t>Best_Design_Cost_Margin_Pct</t>
         </is>
       </c>
       <c r="B12" s="43" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="n"/>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C12" s="51" t="inlineStr">
+        <is>
+          <t>Best design (default): the design with fewer switches and uplinks is kept unless it costs more than this % above the lowest-cost valid design</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
         <is>
-          <t>Default_PoE_Headroom_Pct</t>
+          <t>Default_Spare_Pct</t>
         </is>
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C13" s="43" t="n"/>
@@ -2886,134 +2891,164 @@
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
         <is>
-          <t>Default_Oversubscription</t>
+          <t>Default_PoE_Headroom_Pct</t>
         </is>
       </c>
       <c r="B14" s="43" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>1 = line-rate</t>
-        </is>
-      </c>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="n"/>
     </row>
     <row r="15" ht="23.85" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
         <is>
-          <t>Max_LAG_Members</t>
+          <t>Default_Oversubscription</t>
         </is>
       </c>
       <c r="B15" s="43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" s="43" t="inlineStr">
         <is>
-          <t>Max uplinks per switch</t>
+          <t>1 = line-rate</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
         <is>
-          <t>Min_Uplink_Gbps</t>
+          <t>Max_LAG_Members</t>
         </is>
       </c>
       <c r="B16" s="43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>Slowest uplink speed to the core. 1 allows 1G uplinks when the bandwidth fits (for example audio on stream bandwidth); raise to 10 to force 10G uplinks everywhere</t>
+          <t>Max uplinks per switch</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
         <is>
-          <t>Stream_Uplink_Headroom_Pct</t>
+          <t>Min_Uplink_Gbps</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C17" s="43" t="inlineStr">
         <is>
-          <t>Stream bandwidth basis only: uplinks must carry the stream total plus this margin, because stream rates are typical, not peak. Line-rate needs no margin</t>
+          <t>Slowest uplink speed to the core. 1 allows 1G uplinks when the bandwidth fits (for example audio on stream bandwidth); raise to 10 to force 10G uplinks everywhere</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
         <is>
-          <t>Uplink_LAG_Sizes</t>
+          <t>Stream_Uplink_Headroom_Pct</t>
         </is>
       </c>
       <c r="B18" s="43" t="inlineStr">
         <is>
-          <t>1,2,4,8</t>
-        </is>
-      </c>
-      <c r="C18" s="51" t="inlineStr">
-        <is>
-          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Stream bandwidth basis only: uplinks must carry the stream total plus this margin, because stream rates are typical, not peak. Line-rate needs no margin</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
         <is>
-          <t>In_Rack_Max_m</t>
+          <t>Uplink_LAG_Sizes</t>
         </is>
       </c>
       <c r="B19" s="43" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C19" s="43" t="inlineStr">
-        <is>
-          <t>MDF links at or below this use DAC/AOC</t>
+          <t>1,2,4,8</t>
+        </is>
+      </c>
+      <c r="C19" s="51" t="inlineStr">
+        <is>
+          <t>Allowed uplink counts per LAG. Powers of 2 hash evenly; 1 only when single uplink is allowed</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
         <is>
-          <t>Copper_10G_Max_m</t>
+          <t>In_Rack_Max_m</t>
         </is>
       </c>
       <c r="B20" s="43" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C20" s="43" t="inlineStr">
         <is>
-          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+          <t>MDF links at or below this use DAC/AOC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="43" t="inlineStr">
         <is>
+          <t>Allow_Third_Party_Optics</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="inlineStr">
+        <is>
+          <t>Yes: when no catalog optic reaches the distance but a third-party module type does (25G/100G eSR on multimode up to 300 m, ER/ZR on single mode), it is a valid part in the BoM with a warning. No: treat it as a placeholder and avoid it</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="inlineStr">
+        <is>
+          <t>Copper_10G_Max_m</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>Longest Cat6a run for 10GBASE-T. Used when the gateway router connects to a room switch over copper (core has no free 10G port)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
           <t>Endpoint_Speeds_Gbps</t>
         </is>
       </c>
-      <c r="B21" s="43" t="inlineStr">
+      <c r="B23" s="43" t="inlineStr">
         <is>
           <t>1,2.5,5,10,25,50,100</t>
         </is>
       </c>
-      <c r="C21" s="43" t="inlineStr">
+      <c r="C23" s="43" t="inlineStr">
         <is>
           <t>Speeds offered in the endpoint library</t>
         </is>
@@ -3039,7 +3074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="28" min="1" max="1"/>
@@ -6517,6 +6552,30 @@
       <c r="F120" s="51" t="inlineStr">
         <is>
           <t>Notes on the cost index (no sources published)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="43" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B121" s="51" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C121" s="43" t="n"/>
+      <c r="D121" s="43" t="n"/>
+      <c r="E121" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F121" s="51" t="inlineStr">
+        <is>
+          <t>Maker of the part, shown in the BoM: NETGEAR, optic.ca, or another supplier's name for third-party parts</t>
         </is>
       </c>
     </row>
@@ -24506,7 +24565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S131"/>
+  <dimension ref="A1:T131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="28" min="1" max="1"/>
@@ -24526,6 +24585,7 @@
     <col width="34" customWidth="1" style="28" min="17" max="17"/>
     <col width="14" customWidth="1" style="29" min="18" max="18"/>
     <col width="40" customWidth="1" style="29" min="19" max="19"/>
+    <col width="14" customWidth="1" style="29" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -24636,6 +24696,11 @@
       <c r="S4" s="42" t="inlineStr">
         <is>
           <t>Cost_Note</t>
+        </is>
+      </c>
+      <c r="T4" s="42" t="inlineStr">
+        <is>
+          <t>Brand</t>
         </is>
       </c>
     </row>
@@ -24705,6 +24770,11 @@
         <v>1370</v>
       </c>
       <c r="S5" s="43" t="n"/>
+      <c r="T5" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -24772,6 +24842,11 @@
         <v>2880</v>
       </c>
       <c r="S6" s="43" t="n"/>
+      <c r="T6" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.85" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -24843,6 +24918,11 @@
         <v>1370</v>
       </c>
       <c r="S7" s="43" t="n"/>
+      <c r="T7" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -24910,6 +24990,11 @@
         <v>3600</v>
       </c>
       <c r="S8" s="43" t="n"/>
+      <c r="T8" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -24979,6 +25064,11 @@
       </c>
       <c r="R9" s="43" t="n"/>
       <c r="S9" s="43" t="n"/>
+      <c r="T9" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -25046,6 +25136,11 @@
         <v>8630</v>
       </c>
       <c r="S10" s="43" t="n"/>
+      <c r="T10" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -25115,6 +25210,11 @@
       </c>
       <c r="R11" s="43" t="n"/>
       <c r="S11" s="43" t="n"/>
+      <c r="T11" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -25182,6 +25282,11 @@
         <v>3600</v>
       </c>
       <c r="S12" s="43" t="n"/>
+      <c r="T12" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -25249,6 +25354,11 @@
         <v>3600</v>
       </c>
       <c r="S13" s="43" t="n"/>
+      <c r="T13" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -25316,6 +25426,11 @@
         <v>3430</v>
       </c>
       <c r="S14" s="43" t="n"/>
+      <c r="T14" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -25379,6 +25494,11 @@
         <v>535</v>
       </c>
       <c r="S15" s="43" t="n"/>
+      <c r="T15" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -25442,6 +25562,11 @@
         <v>802</v>
       </c>
       <c r="S16" s="43" t="n"/>
+      <c r="T16" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -25505,6 +25630,11 @@
         <v>1070</v>
       </c>
       <c r="S17" s="43" t="n"/>
+      <c r="T17" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -25568,6 +25698,11 @@
         <v>396</v>
       </c>
       <c r="S18" s="43" t="n"/>
+      <c r="T18" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="29">
       <c r="A19" s="43" t="inlineStr">
@@ -25631,6 +25766,11 @@
         <v>428</v>
       </c>
       <c r="S19" s="43" t="n"/>
+      <c r="T19" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="29">
       <c r="A20" s="43" t="inlineStr">
@@ -25694,6 +25834,11 @@
         <v>503</v>
       </c>
       <c r="S20" s="43" t="n"/>
+      <c r="T20" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="29">
       <c r="A21" s="43" t="inlineStr">
@@ -25757,6 +25902,11 @@
         <v>588</v>
       </c>
       <c r="S21" s="43" t="n"/>
+      <c r="T21" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="46.25" customHeight="1" s="29">
       <c r="A22" s="43" t="inlineStr">
@@ -25820,6 +25970,11 @@
         <v>2900</v>
       </c>
       <c r="S22" s="43" t="n"/>
+      <c r="T22" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="46.25" customHeight="1" s="29">
       <c r="A23" s="43" t="inlineStr">
@@ -25883,6 +26038,11 @@
         <v>2900</v>
       </c>
       <c r="S23" s="43" t="n"/>
+      <c r="T23" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="46.25" customHeight="1" s="29">
       <c r="A24" s="43" t="inlineStr">
@@ -25946,6 +26106,11 @@
         <v>2900</v>
       </c>
       <c r="S24" s="43" t="n"/>
+      <c r="T24" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="46.25" customHeight="1" s="29">
       <c r="A25" s="43" t="inlineStr">
@@ -26009,6 +26174,11 @@
         <v>2900</v>
       </c>
       <c r="S25" s="43" t="n"/>
+      <c r="T25" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="46.25" customHeight="1" s="29">
       <c r="A26" s="43" t="inlineStr">
@@ -26072,6 +26242,11 @@
         <v>3390</v>
       </c>
       <c r="S26" s="43" t="n"/>
+      <c r="T26" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="46.25" customHeight="1" s="29">
       <c r="A27" s="43" t="inlineStr">
@@ -26135,6 +26310,11 @@
         <v>3390</v>
       </c>
       <c r="S27" s="43" t="n"/>
+      <c r="T27" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="46.25" customHeight="1" s="29">
       <c r="A28" s="43" t="inlineStr">
@@ -26198,6 +26378,11 @@
         <v>3390</v>
       </c>
       <c r="S28" s="43" t="n"/>
+      <c r="T28" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="46.25" customHeight="1" s="29">
       <c r="A29" s="43" t="inlineStr">
@@ -26261,6 +26446,11 @@
         <v>4360</v>
       </c>
       <c r="S29" s="43" t="n"/>
+      <c r="T29" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="46.25" customHeight="1" s="29">
       <c r="A30" s="43" t="inlineStr">
@@ -26324,6 +26514,11 @@
         <v>4360</v>
       </c>
       <c r="S30" s="43" t="n"/>
+      <c r="T30" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="46.25" customHeight="1" s="29">
       <c r="A31" s="43" t="inlineStr">
@@ -26387,6 +26582,11 @@
         <v>4360</v>
       </c>
       <c r="S31" s="43" t="n"/>
+      <c r="T31" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="46.25" customHeight="1" s="29">
       <c r="A32" s="43" t="inlineStr">
@@ -26450,6 +26650,11 @@
         <v>7260</v>
       </c>
       <c r="S32" s="43" t="n"/>
+      <c r="T32" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="46.25" customHeight="1" s="29">
       <c r="A33" s="43" t="inlineStr">
@@ -26513,6 +26718,11 @@
         <v>7260</v>
       </c>
       <c r="S33" s="43" t="n"/>
+      <c r="T33" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="46.25" customHeight="1" s="29">
       <c r="A34" s="43" t="inlineStr">
@@ -26576,6 +26786,11 @@
         <v>7260</v>
       </c>
       <c r="S34" s="43" t="n"/>
+      <c r="T34" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="46.25" customHeight="1" s="29">
       <c r="A35" s="43" t="inlineStr">
@@ -26639,6 +26854,11 @@
         <v>3390</v>
       </c>
       <c r="S35" s="43" t="n"/>
+      <c r="T35" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="46.25" customHeight="1" s="29">
       <c r="A36" s="43" t="inlineStr">
@@ -26702,6 +26922,11 @@
         <v>3390</v>
       </c>
       <c r="S36" s="43" t="n"/>
+      <c r="T36" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="46.25" customHeight="1" s="29">
       <c r="A37" s="43" t="inlineStr">
@@ -26765,6 +26990,11 @@
         <v>3390</v>
       </c>
       <c r="S37" s="43" t="n"/>
+      <c r="T37" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="46.25" customHeight="1" s="29">
       <c r="A38" s="43" t="inlineStr">
@@ -26828,6 +27058,11 @@
         <v>4360</v>
       </c>
       <c r="S38" s="43" t="n"/>
+      <c r="T38" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="46.25" customHeight="1" s="29">
       <c r="A39" s="43" t="inlineStr">
@@ -26891,6 +27126,11 @@
         <v>4360</v>
       </c>
       <c r="S39" s="43" t="n"/>
+      <c r="T39" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="46.25" customHeight="1" s="29">
       <c r="A40" s="43" t="inlineStr">
@@ -26954,6 +27194,11 @@
         <v>4360</v>
       </c>
       <c r="S40" s="43" t="n"/>
+      <c r="T40" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="46.25" customHeight="1" s="29">
       <c r="A41" s="43" t="inlineStr">
@@ -27017,6 +27262,11 @@
         <v>7260</v>
       </c>
       <c r="S41" s="43" t="n"/>
+      <c r="T41" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="46.25" customHeight="1" s="29">
       <c r="A42" s="43" t="inlineStr">
@@ -27080,6 +27330,11 @@
         <v>7260</v>
       </c>
       <c r="S42" s="43" t="n"/>
+      <c r="T42" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="46.25" customHeight="1" s="29">
       <c r="A43" s="43" t="inlineStr">
@@ -27143,6 +27398,11 @@
         <v>7260</v>
       </c>
       <c r="S43" s="43" t="n"/>
+      <c r="T43" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="46.25" customHeight="1" s="29">
       <c r="A44" s="43" t="inlineStr">
@@ -27186,6 +27446,11 @@
         <v>2900</v>
       </c>
       <c r="S44" s="43" t="n"/>
+      <c r="T44" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="29">
       <c r="A45" s="43" t="inlineStr">
@@ -27233,6 +27498,11 @@
       </c>
       <c r="R45" s="43" t="n"/>
       <c r="S45" s="43" t="n"/>
+      <c r="T45" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="29">
       <c r="A46" s="43" t="inlineStr">
@@ -27280,6 +27550,11 @@
       </c>
       <c r="R46" s="43" t="n"/>
       <c r="S46" s="43" t="n"/>
+      <c r="T46" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="29">
       <c r="A47" s="43" t="inlineStr">
@@ -27327,6 +27602,11 @@
       </c>
       <c r="R47" s="43" t="n"/>
       <c r="S47" s="43" t="n"/>
+      <c r="T47" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="29">
       <c r="A48" s="43" t="inlineStr">
@@ -27374,6 +27654,11 @@
       </c>
       <c r="R48" s="43" t="n"/>
       <c r="S48" s="43" t="n"/>
+      <c r="T48" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="23.85" customHeight="1" s="29">
       <c r="A49" s="43" t="inlineStr">
@@ -27419,6 +27704,11 @@
       </c>
       <c r="R49" s="43" t="n"/>
       <c r="S49" s="43" t="n"/>
+      <c r="T49" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="23.85" customHeight="1" s="29">
       <c r="A50" s="43" t="inlineStr">
@@ -27466,6 +27756,11 @@
       </c>
       <c r="R50" s="43" t="n"/>
       <c r="S50" s="43" t="n"/>
+      <c r="T50" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="23.85" customHeight="1" s="29">
       <c r="A51" s="43" t="inlineStr">
@@ -27513,6 +27808,11 @@
       </c>
       <c r="R51" s="43" t="n"/>
       <c r="S51" s="43" t="n"/>
+      <c r="T51" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="23.85" customHeight="1" s="29">
       <c r="A52" s="43" t="inlineStr">
@@ -27560,6 +27860,11 @@
       </c>
       <c r="R52" s="43" t="n"/>
       <c r="S52" s="43" t="n"/>
+      <c r="T52" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="29">
       <c r="A53" s="43" t="inlineStr">
@@ -27607,6 +27912,11 @@
       </c>
       <c r="R53" s="43" t="n"/>
       <c r="S53" s="43" t="n"/>
+      <c r="T53" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="29">
       <c r="A54" s="43" t="inlineStr">
@@ -27654,6 +27964,11 @@
       </c>
       <c r="R54" s="43" t="n"/>
       <c r="S54" s="43" t="n"/>
+      <c r="T54" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="29">
       <c r="A55" s="43" t="inlineStr">
@@ -27701,6 +28016,11 @@
       </c>
       <c r="R55" s="43" t="n"/>
       <c r="S55" s="43" t="n"/>
+      <c r="T55" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="46.25" customHeight="1" s="29">
       <c r="A56" s="43" t="inlineStr">
@@ -27748,6 +28068,11 @@
       </c>
       <c r="R56" s="43" t="n"/>
       <c r="S56" s="43" t="n"/>
+      <c r="T56" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="46.25" customHeight="1" s="29">
       <c r="A57" s="43" t="inlineStr">
@@ -27795,6 +28120,11 @@
       </c>
       <c r="R57" s="43" t="n"/>
       <c r="S57" s="43" t="n"/>
+      <c r="T57" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="46.25" customHeight="1" s="29">
       <c r="A58" s="43" t="inlineStr">
@@ -27842,6 +28172,11 @@
       </c>
       <c r="R58" s="43" t="n"/>
       <c r="S58" s="43" t="n"/>
+      <c r="T58" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="29">
       <c r="A59" s="43" t="inlineStr">
@@ -27885,6 +28220,11 @@
       <c r="Q59" s="43" t="n"/>
       <c r="R59" s="43" t="n"/>
       <c r="S59" s="43" t="n"/>
+      <c r="T59" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="29">
       <c r="A60" s="43" t="inlineStr">
@@ -27928,6 +28268,11 @@
       <c r="Q60" s="43" t="n"/>
       <c r="R60" s="43" t="n"/>
       <c r="S60" s="43" t="n"/>
+      <c r="T60" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="29">
       <c r="A61" s="43" t="inlineStr">
@@ -27971,6 +28316,11 @@
       <c r="Q61" s="43" t="n"/>
       <c r="R61" s="43" t="n"/>
       <c r="S61" s="43" t="n"/>
+      <c r="T61" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="23.85" customHeight="1" s="29">
       <c r="A62" s="43" t="inlineStr">
@@ -28014,6 +28364,11 @@
       <c r="Q62" s="43" t="n"/>
       <c r="R62" s="43" t="n"/>
       <c r="S62" s="43" t="n"/>
+      <c r="T62" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="23.85" customHeight="1" s="29">
       <c r="A63" s="43" t="inlineStr">
@@ -28057,6 +28412,11 @@
       <c r="Q63" s="43" t="n"/>
       <c r="R63" s="43" t="n"/>
       <c r="S63" s="43" t="n"/>
+      <c r="T63" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="23.85" customHeight="1" s="29">
       <c r="A64" s="43" t="inlineStr">
@@ -28100,6 +28460,11 @@
       <c r="Q64" s="43" t="n"/>
       <c r="R64" s="43" t="n"/>
       <c r="S64" s="43" t="n"/>
+      <c r="T64" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="29">
       <c r="A65" s="43" t="inlineStr">
@@ -28143,6 +28508,11 @@
       <c r="Q65" s="43" t="n"/>
       <c r="R65" s="43" t="n"/>
       <c r="S65" s="43" t="n"/>
+      <c r="T65" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="29">
       <c r="A66" s="43" t="inlineStr">
@@ -28186,6 +28556,11 @@
       <c r="Q66" s="43" t="n"/>
       <c r="R66" s="43" t="n"/>
       <c r="S66" s="43" t="n"/>
+      <c r="T66" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="29">
       <c r="A67" s="43" t="inlineStr">
@@ -28229,6 +28604,11 @@
       <c r="Q67" s="43" t="n"/>
       <c r="R67" s="43" t="n"/>
       <c r="S67" s="43" t="n"/>
+      <c r="T67" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="23.85" customHeight="1" s="29">
       <c r="A68" s="43" t="inlineStr">
@@ -28272,6 +28652,11 @@
       <c r="Q68" s="43" t="n"/>
       <c r="R68" s="43" t="n"/>
       <c r="S68" s="43" t="n"/>
+      <c r="T68" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="23.85" customHeight="1" s="29">
       <c r="A69" s="43" t="inlineStr">
@@ -28315,6 +28700,11 @@
       <c r="Q69" s="43" t="n"/>
       <c r="R69" s="43" t="n"/>
       <c r="S69" s="43" t="n"/>
+      <c r="T69" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="23.85" customHeight="1" s="29">
       <c r="A70" s="43" t="inlineStr">
@@ -28358,6 +28748,11 @@
       <c r="Q70" s="43" t="n"/>
       <c r="R70" s="43" t="n"/>
       <c r="S70" s="43" t="n"/>
+      <c r="T70" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="23.85" customHeight="1" s="29">
       <c r="A71" s="43" t="inlineStr">
@@ -28429,6 +28824,11 @@
         <v>3510</v>
       </c>
       <c r="S71" s="43" t="n"/>
+      <c r="T71" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="23.85" customHeight="1" s="29">
       <c r="A72" s="43" t="inlineStr">
@@ -28500,6 +28900,11 @@
         <v>8050</v>
       </c>
       <c r="S72" s="43" t="n"/>
+      <c r="T72" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="23.85" customHeight="1" s="29">
       <c r="A73" s="43" t="inlineStr">
@@ -28571,6 +28976,11 @@
         <v>7300</v>
       </c>
       <c r="S73" s="43" t="n"/>
+      <c r="T73" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="23.85" customHeight="1" s="29">
       <c r="A74" s="43" t="inlineStr">
@@ -28642,6 +29052,11 @@
         <v>6820</v>
       </c>
       <c r="S74" s="43" t="n"/>
+      <c r="T74" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="23.85" customHeight="1" s="29">
       <c r="A75" s="43" t="inlineStr">
@@ -28713,6 +29128,11 @@
         <v>6820</v>
       </c>
       <c r="S75" s="43" t="n"/>
+      <c r="T75" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="23.85" customHeight="1" s="29">
       <c r="A76" s="43" t="inlineStr">
@@ -28780,6 +29200,11 @@
         <v>458</v>
       </c>
       <c r="S76" s="43" t="n"/>
+      <c r="T76" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="23.85" customHeight="1" s="29">
       <c r="A77" s="43" t="inlineStr">
@@ -28847,6 +29272,11 @@
         <v>458</v>
       </c>
       <c r="S77" s="43" t="n"/>
+      <c r="T77" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="23.85" customHeight="1" s="29">
       <c r="A78" s="43" t="inlineStr">
@@ -28914,6 +29344,11 @@
         <v>458</v>
       </c>
       <c r="S78" s="43" t="n"/>
+      <c r="T78" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="23.85" customHeight="1" s="29">
       <c r="A79" s="43" t="inlineStr">
@@ -28981,6 +29416,11 @@
         <v>695</v>
       </c>
       <c r="S79" s="43" t="n"/>
+      <c r="T79" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="23.85" customHeight="1" s="29">
       <c r="A80" s="43" t="inlineStr">
@@ -29048,6 +29488,11 @@
         <v>1480</v>
       </c>
       <c r="S80" s="43" t="n"/>
+      <c r="T80" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="23.85" customHeight="1" s="29">
       <c r="A81" s="43" t="inlineStr">
@@ -29115,6 +29560,11 @@
         <v>1480</v>
       </c>
       <c r="S81" s="43" t="n"/>
+      <c r="T81" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="23.85" customHeight="1" s="29">
       <c r="A82" s="43" t="inlineStr">
@@ -29182,6 +29632,11 @@
         <v>1480</v>
       </c>
       <c r="S82" s="43" t="n"/>
+      <c r="T82" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="23.85" customHeight="1" s="29">
       <c r="A83" s="43" t="inlineStr">
@@ -29249,6 +29704,11 @@
         <v>1830</v>
       </c>
       <c r="S83" s="43" t="n"/>
+      <c r="T83" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="23.85" customHeight="1" s="29">
       <c r="A84" s="43" t="inlineStr">
@@ -29316,6 +29776,11 @@
         <v>1830</v>
       </c>
       <c r="S84" s="43" t="n"/>
+      <c r="T84" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="23.85" customHeight="1" s="29">
       <c r="A85" s="43" t="inlineStr">
@@ -29383,6 +29848,11 @@
         <v>1830</v>
       </c>
       <c r="S85" s="43" t="n"/>
+      <c r="T85" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="23.85" customHeight="1" s="29">
       <c r="A86" s="43" t="inlineStr">
@@ -29450,6 +29920,11 @@
         <v>1190</v>
       </c>
       <c r="S86" s="43" t="n"/>
+      <c r="T86" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="23.85" customHeight="1" s="29">
       <c r="A87" s="43" t="inlineStr">
@@ -29517,6 +29992,11 @@
         <v>1190</v>
       </c>
       <c r="S87" s="43" t="n"/>
+      <c r="T87" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="23.85" customHeight="1" s="29">
       <c r="A88" s="43" t="inlineStr">
@@ -29584,6 +30064,11 @@
         <v>1190</v>
       </c>
       <c r="S88" s="43" t="n"/>
+      <c r="T88" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="23.85" customHeight="1" s="29">
       <c r="A89" s="43" t="inlineStr">
@@ -29651,6 +30136,11 @@
         <v>1620</v>
       </c>
       <c r="S89" s="43" t="n"/>
+      <c r="T89" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="23.85" customHeight="1" s="29">
       <c r="A90" s="43" t="inlineStr">
@@ -29718,6 +30208,11 @@
         <v>7030</v>
       </c>
       <c r="S90" s="43" t="n"/>
+      <c r="T90" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="23.85" customHeight="1" s="29">
       <c r="A91" s="43" t="inlineStr">
@@ -29785,6 +30280,11 @@
         <v>7030</v>
       </c>
       <c r="S91" s="43" t="n"/>
+      <c r="T91" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="23.85" customHeight="1" s="29">
       <c r="A92" s="43" t="inlineStr">
@@ -29852,6 +30352,11 @@
         <v>7030</v>
       </c>
       <c r="S92" s="43" t="n"/>
+      <c r="T92" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="23.85" customHeight="1" s="29">
       <c r="A93" s="43" t="inlineStr">
@@ -29919,6 +30424,11 @@
         <v>7740</v>
       </c>
       <c r="S93" s="43" t="n"/>
+      <c r="T93" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="23.85" customHeight="1" s="29">
       <c r="A94" s="43" t="inlineStr">
@@ -29986,6 +30496,11 @@
         <v>7740</v>
       </c>
       <c r="S94" s="43" t="n"/>
+      <c r="T94" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="23.85" customHeight="1" s="29">
       <c r="A95" s="43" t="inlineStr">
@@ -30053,6 +30568,11 @@
         <v>7740</v>
       </c>
       <c r="S95" s="43" t="n"/>
+      <c r="T95" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="23.85" customHeight="1" s="29">
       <c r="A96" s="43" t="inlineStr">
@@ -30120,6 +30640,11 @@
         <v>1670</v>
       </c>
       <c r="S96" s="43" t="n"/>
+      <c r="T96" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="23.85" customHeight="1" s="29">
       <c r="A97" s="43" t="inlineStr">
@@ -30187,6 +30712,11 @@
         <v>1670</v>
       </c>
       <c r="S97" s="43" t="n"/>
+      <c r="T97" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="23.85" customHeight="1" s="29">
       <c r="A98" s="43" t="inlineStr">
@@ -30254,6 +30784,11 @@
         <v>1670</v>
       </c>
       <c r="S98" s="43" t="n"/>
+      <c r="T98" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="23.85" customHeight="1" s="29">
       <c r="A99" s="43" t="inlineStr">
@@ -30321,6 +30856,11 @@
         <v>2470</v>
       </c>
       <c r="S99" s="43" t="n"/>
+      <c r="T99" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="23.85" customHeight="1" s="29">
       <c r="A100" s="43" t="inlineStr">
@@ -30388,6 +30928,11 @@
         <v>7030</v>
       </c>
       <c r="S100" s="43" t="n"/>
+      <c r="T100" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="23.85" customHeight="1" s="29">
       <c r="A101" s="43" t="inlineStr">
@@ -30455,6 +31000,11 @@
         <v>7030</v>
       </c>
       <c r="S101" s="43" t="n"/>
+      <c r="T101" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="23.85" customHeight="1" s="29">
       <c r="A102" s="43" t="inlineStr">
@@ -30522,6 +31072,11 @@
         <v>7030</v>
       </c>
       <c r="S102" s="43" t="n"/>
+      <c r="T102" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="23.85" customHeight="1" s="29">
       <c r="A103" s="43" t="inlineStr">
@@ -30589,6 +31144,11 @@
         <v>7740</v>
       </c>
       <c r="S103" s="43" t="n"/>
+      <c r="T103" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="23.85" customHeight="1" s="29">
       <c r="A104" s="43" t="inlineStr">
@@ -30656,6 +31216,11 @@
         <v>7740</v>
       </c>
       <c r="S104" s="43" t="n"/>
+      <c r="T104" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="23.85" customHeight="1" s="29">
       <c r="A105" s="43" t="inlineStr">
@@ -30723,6 +31288,11 @@
         <v>7740</v>
       </c>
       <c r="S105" s="43" t="n"/>
+      <c r="T105" s="43" t="inlineStr">
+        <is>
+          <t>optic.ca</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="23.85" customHeight="1" s="29">
       <c r="A106" s="43" t="inlineStr">
@@ -30792,6 +31362,11 @@
       </c>
       <c r="R106" s="43" t="n"/>
       <c r="S106" s="43" t="n"/>
+      <c r="T106" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="23.85" customHeight="1" s="29">
       <c r="A107" s="43" t="inlineStr">
@@ -30861,6 +31436,11 @@
       </c>
       <c r="R107" s="43" t="n"/>
       <c r="S107" s="43" t="n"/>
+      <c r="T107" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="23.85" customHeight="1" s="29">
       <c r="A108" s="43" t="inlineStr">
@@ -30926,6 +31506,11 @@
       <c r="Q108" s="43" t="n"/>
       <c r="R108" s="43" t="n"/>
       <c r="S108" s="43" t="n"/>
+      <c r="T108" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="23.85" customHeight="1" s="29">
       <c r="A109" s="43" t="inlineStr">
@@ -30991,6 +31576,11 @@
       <c r="Q109" s="43" t="n"/>
       <c r="R109" s="43" t="n"/>
       <c r="S109" s="43" t="n"/>
+      <c r="T109" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="23.85" customHeight="1" s="29">
       <c r="A110" s="43" t="inlineStr">
@@ -31052,6 +31642,11 @@
       <c r="Q110" s="43" t="n"/>
       <c r="R110" s="43" t="n"/>
       <c r="S110" s="43" t="n"/>
+      <c r="T110" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="23.85" customHeight="1" s="29">
       <c r="A111" s="43" t="inlineStr">
@@ -31113,6 +31708,11 @@
       <c r="Q111" s="43" t="n"/>
       <c r="R111" s="43" t="n"/>
       <c r="S111" s="43" t="n"/>
+      <c r="T111" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="23.85" customHeight="1" s="29">
       <c r="A112" s="43" t="inlineStr">
@@ -31174,6 +31774,11 @@
       <c r="Q112" s="43" t="n"/>
       <c r="R112" s="43" t="n"/>
       <c r="S112" s="43" t="n"/>
+      <c r="T112" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="23.85" customHeight="1" s="29">
       <c r="A113" s="43" t="inlineStr">
@@ -31235,6 +31840,11 @@
       <c r="Q113" s="43" t="n"/>
       <c r="R113" s="43" t="n"/>
       <c r="S113" s="43" t="n"/>
+      <c r="T113" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="23.85" customHeight="1" s="29">
       <c r="A114" s="43" t="inlineStr">
@@ -31292,6 +31902,11 @@
       </c>
       <c r="R114" s="43" t="n"/>
       <c r="S114" s="43" t="n"/>
+      <c r="T114" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="23.85" customHeight="1" s="29">
       <c r="A115" s="43" t="inlineStr">
@@ -31341,6 +31956,11 @@
       </c>
       <c r="R115" s="43" t="n"/>
       <c r="S115" s="43" t="n"/>
+      <c r="T115" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="23.85" customHeight="1" s="29">
       <c r="A116" s="43" t="inlineStr">
@@ -31388,6 +32008,11 @@
       </c>
       <c r="R116" s="43" t="n"/>
       <c r="S116" s="43" t="n"/>
+      <c r="T116" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="23.85" customHeight="1" s="29">
       <c r="A117" s="43" t="inlineStr">
@@ -31435,6 +32060,11 @@
       </c>
       <c r="R117" s="43" t="n"/>
       <c r="S117" s="43" t="n"/>
+      <c r="T117" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="23.85" customHeight="1" s="29">
       <c r="A118" s="43" t="inlineStr">
@@ -31482,6 +32112,11 @@
       </c>
       <c r="R118" s="43" t="n"/>
       <c r="S118" s="43" t="n"/>
+      <c r="T118" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="23.85" customHeight="1" s="29">
       <c r="A119" s="43" t="inlineStr">
@@ -31525,6 +32160,11 @@
       <c r="Q119" s="43" t="n"/>
       <c r="R119" s="43" t="n"/>
       <c r="S119" s="43" t="n"/>
+      <c r="T119" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="23.85" customHeight="1" s="29">
       <c r="A120" s="43" t="inlineStr">
@@ -31568,6 +32208,11 @@
       <c r="Q120" s="43" t="n"/>
       <c r="R120" s="43" t="n"/>
       <c r="S120" s="43" t="n"/>
+      <c r="T120" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="23.85" customHeight="1" s="29">
       <c r="A121" s="43" t="inlineStr">
@@ -31611,6 +32256,11 @@
       <c r="Q121" s="43" t="n"/>
       <c r="R121" s="43" t="n"/>
       <c r="S121" s="43" t="n"/>
+      <c r="T121" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="23.85" customHeight="1" s="29">
       <c r="A122" s="43" t="inlineStr">
@@ -31658,6 +32308,11 @@
       </c>
       <c r="R122" s="43" t="n"/>
       <c r="S122" s="43" t="n"/>
+      <c r="T122" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="23.85" customHeight="1" s="29">
       <c r="A123" s="43" t="inlineStr">
@@ -31705,6 +32360,11 @@
       </c>
       <c r="R123" s="43" t="n"/>
       <c r="S123" s="43" t="n"/>
+      <c r="T123" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="23.85" customHeight="1" s="29">
       <c r="A124" s="43" t="inlineStr">
@@ -31752,6 +32412,11 @@
       </c>
       <c r="R124" s="43" t="n"/>
       <c r="S124" s="43" t="n"/>
+      <c r="T124" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="23.85" customHeight="1" s="29">
       <c r="A125" s="43" t="inlineStr">
@@ -31795,6 +32460,11 @@
       <c r="Q125" s="43" t="n"/>
       <c r="R125" s="43" t="n"/>
       <c r="S125" s="43" t="n"/>
+      <c r="T125" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="23.85" customHeight="1" s="29">
       <c r="A126" s="43" t="inlineStr">
@@ -31838,6 +32508,11 @@
       <c r="Q126" s="43" t="n"/>
       <c r="R126" s="43" t="n"/>
       <c r="S126" s="43" t="n"/>
+      <c r="T126" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="23.85" customHeight="1" s="29">
       <c r="A127" s="43" t="inlineStr">
@@ -31881,6 +32556,11 @@
       <c r="Q127" s="43" t="n"/>
       <c r="R127" s="43" t="n"/>
       <c r="S127" s="43" t="n"/>
+      <c r="T127" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="23.85" customHeight="1" s="29">
       <c r="A128" s="43" t="inlineStr">
@@ -31940,6 +32620,11 @@
         <v>6420</v>
       </c>
       <c r="S128" s="43" t="n"/>
+      <c r="T128" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="23.85" customHeight="1" s="29">
       <c r="A129" s="43" t="inlineStr">
@@ -31999,6 +32684,11 @@
         <v>6420</v>
       </c>
       <c r="S129" s="43" t="n"/>
+      <c r="T129" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="23.85" customHeight="1" s="29">
       <c r="A130" s="43" t="inlineStr">
@@ -32062,6 +32752,11 @@
         <v>13900</v>
       </c>
       <c r="S130" s="43" t="n"/>
+      <c r="T130" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="23.85" customHeight="1" s="29">
       <c r="A131" s="43" t="inlineStr">
@@ -32125,11 +32820,16 @@
         <v>13900</v>
       </c>
       <c r="S131" s="43" t="n"/>
+      <c r="T131" s="43" t="inlineStr">
+        <is>
+          <t>NETGEAR</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:S2"/>
-    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C5:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">

</xml_diff>

<commit_message>
Add connection modes for devices such as WiFi 7 APs
- Endpoints sheet: Alt_Link_Speeds_Gbps and Reduced_PoE_W / _Label /
  _Note (WBE758: 5G/2.5G/1G, PoE+ with reduced radios; WBE718: 1G, PoE
  802.3af with reduced radios), from the datasheets
- New Connection setting per device line in a room; the engine sizes the
  line as the chosen mode (port speed, PoE class and budget, bandwidth)
  and never downgrades on its own
- Checks warns for reduced radios and for 1G AP backhaul, and notes other
  lower port speeds; BoM keeps the normal AP part number; PDF and Excel
  device lists show the chosen mode
- Add validation scenarios V44 and V45
</commit_message>
<xml_diff>
--- a/catalog/NETGEAR_BoM_Catalog.xlsx
+++ b/catalog/NETGEAR_BoM_Catalog.xlsx
@@ -1161,7 +1161,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tblDictionary" displayName="tblDictionary" ref="A4:F125" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:F113"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Sheet"/>
@@ -1278,9 +1278,9 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblEndpoints" displayName="tblEndpoints" ref="A4:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblEndpoints" displayName="tblEndpoints" ref="A4:N19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A4:J18"/>
-  <tableColumns count="10">
+  <tableColumns count="14">
     <tableColumn id="1" name="Endpoint_ID"/>
     <tableColumn id="2" name="Name"/>
     <tableColumn id="3" name="Category"/>
@@ -1291,6 +1291,10 @@
     <tableColumn id="8" name="NETGEAR_Product_ID"/>
     <tableColumn id="9" name="Notes"/>
     <tableColumn id="10" name="Timing"/>
+    <tableColumn id="11" name="Alt_Link_Speeds_Gbps"/>
+    <tableColumn id="12" name="Reduced_PoE_W"/>
+    <tableColumn id="13" name="Reduced_PoE_Label"/>
+    <tableColumn id="14" name="Reduced_PoE_Note"/>
   </tableColumns>
 </table>
 </file>
@@ -3074,7 +3078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="28" min="1" max="1"/>
@@ -6576,6 +6580,110 @@
       <c r="F121" s="51" t="inlineStr">
         <is>
           <t>Maker of the part, shown in the BoM: NETGEAR, optic.ca, or another supplier's name for third-party parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="43" t="inlineStr">
+        <is>
+          <t>Endpoints</t>
+        </is>
+      </c>
+      <c r="B122" s="51" t="inlineStr">
+        <is>
+          <t>Alt_Link_Speeds_Gbps</t>
+        </is>
+      </c>
+      <c r="C122" s="43" t="n"/>
+      <c r="D122" s="43" t="inlineStr">
+        <is>
+          <t>Gbps</t>
+        </is>
+      </c>
+      <c r="E122" s="43" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="F122" s="51" t="inlineStr">
+        <is>
+          <t>Other port speeds the device can run at (e.g. a 10G multi-gig AP on 5G, 2.5G or 1G). Offered as connection options per room</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="43" t="inlineStr">
+        <is>
+          <t>Endpoints</t>
+        </is>
+      </c>
+      <c r="B123" s="51" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_W</t>
+        </is>
+      </c>
+      <c r="C123" s="43" t="n"/>
+      <c r="D123" s="43" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="E123" s="43" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="F123" s="51" t="inlineStr">
+        <is>
+          <t>Power draw in reduced-power mode (lower PoE class). Offered as a connection option</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="43" t="inlineStr">
+        <is>
+          <t>Endpoints</t>
+        </is>
+      </c>
+      <c r="B124" s="51" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_Label</t>
+        </is>
+      </c>
+      <c r="C124" s="43" t="n"/>
+      <c r="D124" s="43" t="n"/>
+      <c r="E124" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F124" s="51" t="inlineStr">
+        <is>
+          <t>PoE class in reduced-power mode, e.g. PoE+ (802.3at)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="43" t="inlineStr">
+        <is>
+          <t>Endpoints</t>
+        </is>
+      </c>
+      <c r="B125" s="51" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_Note</t>
+        </is>
+      </c>
+      <c r="C125" s="43" t="n"/>
+      <c r="D125" s="43" t="n"/>
+      <c r="E125" s="43" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F125" s="51" t="inlineStr">
+        <is>
+          <t>What the device loses in reduced-power mode; shown as a warning in Checks</t>
         </is>
       </c>
     </row>
@@ -45103,7 +45211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="28" min="1" max="1"/>
@@ -45116,6 +45224,10 @@
     <col width="14" customWidth="1" style="28" min="8" max="8"/>
     <col width="44" customWidth="1" style="28" min="9" max="9"/>
     <col width="12" customWidth="1" style="29" min="10" max="10"/>
+    <col width="14" customWidth="1" style="29" min="11" max="11"/>
+    <col width="12" customWidth="1" style="29" min="12" max="12"/>
+    <col width="16" customWidth="1" style="29" min="13" max="13"/>
+    <col width="40" customWidth="1" style="29" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="29">
@@ -45183,6 +45295,26 @@
           <t>Timing</t>
         </is>
       </c>
+      <c r="K4" s="42" t="inlineStr">
+        <is>
+          <t>Alt_Link_Speeds_Gbps</t>
+        </is>
+      </c>
+      <c r="L4" s="42" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_W</t>
+        </is>
+      </c>
+      <c r="M4" s="42" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_Label</t>
+        </is>
+      </c>
+      <c r="N4" s="42" t="inlineStr">
+        <is>
+          <t>Reduced_PoE_Note</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.85" customHeight="1" s="29">
       <c r="A5" s="43" t="inlineStr">
@@ -45221,6 +45353,10 @@
         </is>
       </c>
       <c r="J5" s="51" t="n"/>
+      <c r="K5" s="51" t="n"/>
+      <c r="L5" s="51" t="n"/>
+      <c r="M5" s="51" t="n"/>
+      <c r="N5" s="51" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="29">
       <c r="A6" s="43" t="inlineStr">
@@ -45255,6 +45391,10 @@
       <c r="H6" s="43" t="n"/>
       <c r="I6" s="43" t="n"/>
       <c r="J6" s="43" t="n"/>
+      <c r="K6" s="43" t="n"/>
+      <c r="L6" s="43" t="n"/>
+      <c r="M6" s="43" t="n"/>
+      <c r="N6" s="43" t="n"/>
     </row>
     <row r="7" ht="23.85" customHeight="1" s="29">
       <c r="A7" s="43" t="inlineStr">
@@ -45293,6 +45433,10 @@
         </is>
       </c>
       <c r="J7" s="51" t="n"/>
+      <c r="K7" s="51" t="n"/>
+      <c r="L7" s="51" t="n"/>
+      <c r="M7" s="51" t="n"/>
+      <c r="N7" s="51" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
       <c r="A8" s="43" t="inlineStr">
@@ -45327,6 +45471,10 @@
       <c r="H8" s="43" t="n"/>
       <c r="I8" s="43" t="n"/>
       <c r="J8" s="43" t="n"/>
+      <c r="K8" s="43" t="n"/>
+      <c r="L8" s="43" t="n"/>
+      <c r="M8" s="43" t="n"/>
+      <c r="N8" s="43" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="29">
       <c r="A9" s="43" t="inlineStr">
@@ -45365,6 +45513,10 @@
         </is>
       </c>
       <c r="J9" s="43" t="n"/>
+      <c r="K9" s="43" t="n"/>
+      <c r="L9" s="43" t="n"/>
+      <c r="M9" s="43" t="n"/>
+      <c r="N9" s="43" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="29">
       <c r="A10" s="43" t="inlineStr">
@@ -45407,6 +45559,10 @@
           <t>PTP-BC</t>
         </is>
       </c>
+      <c r="K10" s="43" t="n"/>
+      <c r="L10" s="43" t="n"/>
+      <c r="M10" s="43" t="n"/>
+      <c r="N10" s="43" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="29">
       <c r="A11" s="43" t="inlineStr">
@@ -45441,6 +45597,10 @@
       <c r="H11" s="43" t="n"/>
       <c r="I11" s="43" t="n"/>
       <c r="J11" s="43" t="n"/>
+      <c r="K11" s="43" t="n"/>
+      <c r="L11" s="43" t="n"/>
+      <c r="M11" s="43" t="n"/>
+      <c r="N11" s="43" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="29">
       <c r="A12" s="43" t="inlineStr">
@@ -45475,6 +45635,10 @@
       <c r="H12" s="43" t="n"/>
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="43" t="n"/>
+      <c r="K12" s="43" t="n"/>
+      <c r="L12" s="43" t="n"/>
+      <c r="M12" s="43" t="n"/>
+      <c r="N12" s="43" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="29">
       <c r="A13" s="43" t="inlineStr">
@@ -45509,6 +45673,10 @@
       <c r="H13" s="43" t="n"/>
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="43" t="n"/>
+      <c r="K13" s="43" t="n"/>
+      <c r="L13" s="43" t="n"/>
+      <c r="M13" s="43" t="n"/>
+      <c r="N13" s="43" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="29">
       <c r="A14" s="43" t="inlineStr">
@@ -45543,6 +45711,10 @@
       <c r="H14" s="43" t="n"/>
       <c r="I14" s="43" t="n"/>
       <c r="J14" s="43" t="n"/>
+      <c r="K14" s="43" t="n"/>
+      <c r="L14" s="43" t="n"/>
+      <c r="M14" s="43" t="n"/>
+      <c r="N14" s="43" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="29">
       <c r="A15" s="43" t="inlineStr">
@@ -45577,6 +45749,10 @@
       <c r="H15" s="43" t="n"/>
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="43" t="n"/>
+      <c r="K15" s="43" t="n"/>
+      <c r="L15" s="43" t="n"/>
+      <c r="M15" s="43" t="n"/>
+      <c r="N15" s="43" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="29">
       <c r="A16" s="43" t="inlineStr">
@@ -45619,6 +45795,24 @@
         </is>
       </c>
       <c r="J16" s="43" t="n"/>
+      <c r="K16" s="43" t="inlineStr">
+        <is>
+          <t>5,2.5,1</t>
+        </is>
+      </c>
+      <c r="L16" s="43" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="M16" s="43" t="inlineStr">
+        <is>
+          <t>PoE+ (802.3at)</t>
+        </is>
+      </c>
+      <c r="N16" s="43" t="inlineStr">
+        <is>
+          <t>reduced radios: -50% on 2.4 GHz, -25% on 5 GHz and 6 GHz (802.3af not supported)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="29">
       <c r="A17" s="43" t="inlineStr">
@@ -45661,6 +45855,24 @@
         </is>
       </c>
       <c r="J17" s="43" t="n"/>
+      <c r="K17" s="43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L17" s="43" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="M17" s="43" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="N17" s="43" t="inlineStr">
+        <is>
+          <t>reduced radios: -50% on 2.4 GHz, -25% on 5 GHz, no 6 GHz</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="29">
       <c r="A18" s="43" t="inlineStr">
@@ -45703,6 +45915,10 @@
           <t>AVB</t>
         </is>
       </c>
+      <c r="K18" s="43" t="n"/>
+      <c r="L18" s="43" t="n"/>
+      <c r="M18" s="43" t="n"/>
+      <c r="N18" s="43" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="43" t="inlineStr">
@@ -45745,11 +45961,15 @@
           <t>PTP-BC</t>
         </is>
       </c>
+      <c r="K19" s="43" t="n"/>
+      <c r="L19" s="43" t="n"/>
+      <c r="M19" s="43" t="n"/>
+      <c r="N19" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D5:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">

</xml_diff>